<commit_message>
feat: implement Gemini extraction provider with model fallback and add corresponding tests
</commit_message>
<xml_diff>
--- a/data/GoldenCare_Master.xlsx
+++ b/data/GoldenCare_Master.xlsx
@@ -11,8 +11,8 @@
     <sheet name="שורות חיוב" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'מסמכים'!$A$1:$W$7</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'שורות חיוב'!$A$1:$J$24</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'מסמכים'!$A$1:$W$17</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'שורות חיוב'!$A$1:$J$52</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -39,7 +39,7 @@
       <color rgb="00FFFFFF"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -61,6 +61,11 @@
         <fgColor rgb="00C6EFCE"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFC7CE"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -74,7 +79,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -101,6 +106,9 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -468,7 +476,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:W7"/>
+  <dimension ref="A1:W17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -1063,7 +1071,7 @@
         <v>6</v>
       </c>
       <c r="B7" s="7" t="n">
-        <v>46292.76365407391</v>
+        <v>46292.76365407407</v>
       </c>
       <c r="C7" s="9" t="inlineStr">
         <is>
@@ -1143,8 +1151,883 @@
         </is>
       </c>
     </row>
+    <row r="8">
+      <c r="A8" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" s="7" t="n">
+        <v>46292.76761451389</v>
+      </c>
+      <c r="C8" s="10" t="inlineStr">
+        <is>
+          <t>חילוץ נכשל</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>החילוץ נכשל בכל ספקי ה-AI. פרטים: gemini/-: [Errno 32] Broken pipe</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>מייל נכנס</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>גיא כהן &lt;mail4games21@gmail.com&gt;</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>בדיקת חשבונית (טסט לאוטומציה)</t>
+        </is>
+      </c>
+      <c r="H8" s="2" t="inlineStr">
+        <is>
+          <t>טופס התחשבנות 4 (תקול - חוסר שדות וערכים לא מספריים) - א.ב. מיזוג.pdf</t>
+        </is>
+      </c>
+      <c r="I8" s="2" t="n"/>
+      <c r="J8" s="2" t="n"/>
+      <c r="K8" s="2" t="n"/>
+      <c r="L8" s="2" t="n"/>
+      <c r="M8" s="8" t="n"/>
+      <c r="N8" s="8" t="n"/>
+      <c r="O8" s="8" t="n"/>
+      <c r="P8" s="2" t="n"/>
+      <c r="Q8" s="6" t="n"/>
+      <c r="R8" s="2" t="n"/>
+      <c r="S8" s="6" t="n"/>
+      <c r="T8" s="6" t="n"/>
+      <c r="U8" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="V8" s="2" t="n"/>
+      <c r="W8" s="2" t="inlineStr">
+        <is>
+          <t>פרומפט מומלץ – טופסי התחשבנות v2</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" s="7" t="n">
+        <v>46292.76761696759</v>
+      </c>
+      <c r="C9" s="10" t="inlineStr">
+        <is>
+          <t>חילוץ נכשל</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>החילוץ נכשל בכל ספקי ה-AI. פרטים: gemini/-: [SSL: UNEXPECTED_EOF_WHILE_READING] unexpected eof while reading (_ssl.c:2590)</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>מייל נכנס</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>גיא כהן &lt;mail4games21@gmail.com&gt;</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>בדיקת חשבונית (טסט לאוטומציה)</t>
+        </is>
+      </c>
+      <c r="H9" s="2" t="inlineStr">
+        <is>
+          <t>טופס התחשבנות 2 (תקין - עיצוב שונה) - ש.ל.ה הסעות רפואיות.pdf</t>
+        </is>
+      </c>
+      <c r="I9" s="2" t="n"/>
+      <c r="J9" s="2" t="n"/>
+      <c r="K9" s="2" t="n"/>
+      <c r="L9" s="2" t="n"/>
+      <c r="M9" s="8" t="n"/>
+      <c r="N9" s="8" t="n"/>
+      <c r="O9" s="8" t="n"/>
+      <c r="P9" s="2" t="n"/>
+      <c r="Q9" s="6" t="n"/>
+      <c r="R9" s="2" t="n"/>
+      <c r="S9" s="6" t="n"/>
+      <c r="T9" s="6" t="n"/>
+      <c r="U9" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="V9" s="2" t="n"/>
+      <c r="W9" s="2" t="inlineStr">
+        <is>
+          <t>פרומפט מומלץ – טופסי התחשבנות v2</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" s="7" t="n">
+        <v>46292.76761822917</v>
+      </c>
+      <c r="C10" s="4" t="inlineStr">
+        <is>
+          <t>דורש בדיקה</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>• סכום השורות (14,100.00) שונה מהסה"כ לפני מע"מ (12,500.00)
+• סה"כ לפני מע"מ + מע"מ = 14,625.00, אך הסה"כ לתשלום בטופס הוא 15,625.00</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>מייל נכנס</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>גיא כהן &lt;mail4games21@gmail.com&gt;</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>בדיקת חשבונית (טסט לאוטומציה)</t>
+        </is>
+      </c>
+      <c r="H10" s="2" t="inlineStr">
+        <is>
+          <t>טופס התחשבנות 3 (תקול - אי התאמה בחישוב) - קלין-טק כביסה.pdf</t>
+        </is>
+      </c>
+      <c r="I10" s="2" t="inlineStr">
+        <is>
+          <t>קלין-טק שירותי כביסה וסטריליזציה למוסדות בע"מ</t>
+        </is>
+      </c>
+      <c r="J10" s="2" t="inlineStr">
+        <is>
+          <t>515602119</t>
+        </is>
+      </c>
+      <c r="K10" s="2" t="inlineStr">
+        <is>
+          <t>טופס התחשבנות</t>
+        </is>
+      </c>
+      <c r="L10" s="2" t="inlineStr">
+        <is>
+          <t>CT-2026-409</t>
+        </is>
+      </c>
+      <c r="M10" s="8" t="n">
+        <v>46275</v>
+      </c>
+      <c r="N10" s="8" t="n">
+        <v>46235</v>
+      </c>
+      <c r="O10" s="8" t="n">
+        <v>46265</v>
+      </c>
+      <c r="P10" s="2" t="inlineStr">
+        <is>
+          <t>ILS</t>
+        </is>
+      </c>
+      <c r="Q10" s="6" t="n">
+        <v>12500</v>
+      </c>
+      <c r="R10" s="2" t="n">
+        <v>17</v>
+      </c>
+      <c r="S10" s="6" t="n">
+        <v>2125</v>
+      </c>
+      <c r="T10" s="6" t="n">
+        <v>15625</v>
+      </c>
+      <c r="U10" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="V10" s="2" t="inlineStr">
+        <is>
+          <t>gemini/gemini-3.5-flash-lite</t>
+        </is>
+      </c>
+      <c r="W10" s="2" t="inlineStr">
+        <is>
+          <t>פרומפט מומלץ – טופסי התחשבנות v2</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" s="7" t="n">
+        <v>46292.76812384259</v>
+      </c>
+      <c r="C11" s="4" t="inlineStr">
+        <is>
+          <t>דורש בדיקה</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>• שורה 2: 250 × 16.00 = 4,000.00, אך בטופס מופיע 4,800.00
+• מע"מ 17% על 18,700.00 צריך להיות 3,179.00, אך בטופס מופיע 3,366.00</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>מייל נכנס</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>גיא כהן &lt;mail4games21@gmail.com&gt;</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>בדיקת חשבונית (טסט לאוטומציה)</t>
+        </is>
+      </c>
+      <c r="H11" s="2" t="inlineStr">
+        <is>
+          <t>טופס התחשבנות 5 (תקול - טעות כפל בשורה ומע_מ שגוי) - שפע קייטרינג.pdf</t>
+        </is>
+      </c>
+      <c r="I11" s="2" t="inlineStr">
+        <is>
+          <t>שפע טעמים - הסעדה וקייטרינג למוסדות רפואיים בע"מ</t>
+        </is>
+      </c>
+      <c r="J11" s="2" t="inlineStr">
+        <is>
+          <t>511209844</t>
+        </is>
+      </c>
+      <c r="K11" s="2" t="inlineStr">
+        <is>
+          <t>חשבונית ריכוז</t>
+        </is>
+      </c>
+      <c r="L11" s="2" t="inlineStr">
+        <is>
+          <t>SH-2026-9912</t>
+        </is>
+      </c>
+      <c r="M11" s="8" t="n">
+        <v>46267</v>
+      </c>
+      <c r="N11" s="8" t="n">
+        <v>46235</v>
+      </c>
+      <c r="O11" s="8" t="n">
+        <v>46265</v>
+      </c>
+      <c r="P11" s="2" t="inlineStr">
+        <is>
+          <t>ILS</t>
+        </is>
+      </c>
+      <c r="Q11" s="6" t="n">
+        <v>18700</v>
+      </c>
+      <c r="R11" s="2" t="n">
+        <v>17</v>
+      </c>
+      <c r="S11" s="6" t="n">
+        <v>3366</v>
+      </c>
+      <c r="T11" s="6" t="n">
+        <v>22066</v>
+      </c>
+      <c r="U11" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="V11" s="2" t="inlineStr">
+        <is>
+          <t>gemini/gemini-3.5-flash-lite</t>
+        </is>
+      </c>
+      <c r="W11" s="2" t="inlineStr">
+        <is>
+          <t>פרומפט מומלץ – טופסי התחשבנות v2</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" s="7" t="n">
+        <v>46292.7681909838</v>
+      </c>
+      <c r="C12" s="9" t="inlineStr">
+        <is>
+          <t>תקין</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr"/>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>מייל נכנס</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>גיא כהן &lt;mail4games21@gmail.com&gt;</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>בדיקת חשבונית (טסט לאוטומציה)</t>
+        </is>
+      </c>
+      <c r="H12" s="2" t="inlineStr">
+        <is>
+          <t>טופס התחשבנות ספק - מדי-פארם בע_מ.pdf</t>
+        </is>
+      </c>
+      <c r="I12" s="2" t="inlineStr">
+        <is>
+          <t>מדי-פארם ציוד רפואי וסיעודי בע"מ</t>
+        </is>
+      </c>
+      <c r="J12" s="2" t="inlineStr">
+        <is>
+          <t>514892031</t>
+        </is>
+      </c>
+      <c r="K12" s="2" t="inlineStr">
+        <is>
+          <t>טופס התחשבנות ספק / חשבונית</t>
+        </is>
+      </c>
+      <c r="L12" s="2" t="inlineStr">
+        <is>
+          <t>MP-2026-0894</t>
+        </is>
+      </c>
+      <c r="M12" s="8" t="n">
+        <v>46280</v>
+      </c>
+      <c r="N12" s="8" t="n">
+        <v>46235</v>
+      </c>
+      <c r="O12" s="8" t="n">
+        <v>46265</v>
+      </c>
+      <c r="P12" s="2" t="inlineStr">
+        <is>
+          <t>ILS</t>
+        </is>
+      </c>
+      <c r="Q12" s="6" t="n">
+        <v>16000</v>
+      </c>
+      <c r="R12" s="2" t="n">
+        <v>17</v>
+      </c>
+      <c r="S12" s="6" t="n">
+        <v>2720</v>
+      </c>
+      <c r="T12" s="6" t="n">
+        <v>18720</v>
+      </c>
+      <c r="U12" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="V12" s="2" t="inlineStr">
+        <is>
+          <t>gemini/gemini-3.5-flash-lite</t>
+        </is>
+      </c>
+      <c r="W12" s="2" t="inlineStr">
+        <is>
+          <t>פרומפט מומלץ – טופסי התחשבנות v2</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" s="7" t="n">
+        <v>46292.77518795139</v>
+      </c>
+      <c r="C13" s="4" t="inlineStr">
+        <is>
+          <t>דורש בדיקה</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>• שדה חובה חסר: מספר מסמך
+• שדה חובה חסר: תאריך המסמך
+• שדה חובה חסר: סה"כ לתשלום
+• שורה 3: אין סכום לשורה</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>מייל נכנס</t>
+        </is>
+      </c>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>גיא כהן &lt;mail4games21@gmail.com&gt;</t>
+        </is>
+      </c>
+      <c r="G13" s="2" t="inlineStr">
+        <is>
+          <t>בדיקת חשבונית (טסט לאוטומציה)</t>
+        </is>
+      </c>
+      <c r="H13" s="2" t="inlineStr">
+        <is>
+          <t>טופס התחשבנות 4 (תקול - חוסר שדות וערכים לא מספריים) - א.ב. מיזוג.pdf</t>
+        </is>
+      </c>
+      <c r="I13" s="2" t="inlineStr">
+        <is>
+          <t>א.ב. הנדסת מיזוג אוויר ואחזקת מבנים</t>
+        </is>
+      </c>
+      <c r="J13" s="2" t="inlineStr">
+        <is>
+          <t>039481221</t>
+        </is>
+      </c>
+      <c r="K13" s="2" t="inlineStr">
+        <is>
+          <t>טופס התחשבנות זמני / חסר השלמה</t>
+        </is>
+      </c>
+      <c r="L13" s="2" t="n"/>
+      <c r="M13" s="8" t="n"/>
+      <c r="N13" s="8" t="n"/>
+      <c r="O13" s="8" t="n"/>
+      <c r="P13" s="2" t="inlineStr">
+        <is>
+          <t>ILS</t>
+        </is>
+      </c>
+      <c r="Q13" s="6" t="n">
+        <v>9550</v>
+      </c>
+      <c r="R13" s="2" t="n">
+        <v>17</v>
+      </c>
+      <c r="S13" s="6" t="n"/>
+      <c r="T13" s="6" t="n"/>
+      <c r="U13" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="V13" s="2" t="inlineStr">
+        <is>
+          <t>gemini/gemini-3.5-flash-lite</t>
+        </is>
+      </c>
+      <c r="W13" s="2" t="inlineStr">
+        <is>
+          <t>פרומפט מומלץ – טופסי התחשבנות v2</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" s="7" t="n">
+        <v>46292.77586778935</v>
+      </c>
+      <c r="C14" s="9" t="inlineStr">
+        <is>
+          <t>תקין</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr"/>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>מייל נכנס</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>גיא כהן &lt;mail4games21@gmail.com&gt;</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t>בדיקת חשבונית (טסט לאוטומציה)</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="inlineStr">
+        <is>
+          <t>טופס התחשבנות 2 (תקין - עיצוב שונה) - ש.ל.ה הסעות רפואיות.pdf</t>
+        </is>
+      </c>
+      <c r="I14" s="2" t="inlineStr">
+        <is>
+          <t>ש.ל.ה שירותי לוגיסטיקה והסעות רפואיות בע"מ</t>
+        </is>
+      </c>
+      <c r="J14" s="2" t="inlineStr">
+        <is>
+          <t>512998410</t>
+        </is>
+      </c>
+      <c r="K14" s="2" t="inlineStr">
+        <is>
+          <t>ריכוז חיובים חודשי</t>
+        </is>
+      </c>
+      <c r="L14" s="2" t="inlineStr">
+        <is>
+          <t>SLH-88421</t>
+        </is>
+      </c>
+      <c r="M14" s="8" t="n">
+        <v>46264</v>
+      </c>
+      <c r="N14" s="8" t="n">
+        <v>46235</v>
+      </c>
+      <c r="O14" s="8" t="n">
+        <v>46265</v>
+      </c>
+      <c r="P14" s="2" t="inlineStr">
+        <is>
+          <t>ILS</t>
+        </is>
+      </c>
+      <c r="Q14" s="6" t="n">
+        <v>11000</v>
+      </c>
+      <c r="R14" s="2" t="n">
+        <v>17</v>
+      </c>
+      <c r="S14" s="6" t="n">
+        <v>1870</v>
+      </c>
+      <c r="T14" s="6" t="n">
+        <v>12870</v>
+      </c>
+      <c r="U14" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="V14" s="2" t="inlineStr">
+        <is>
+          <t>gemini/gemini-3.5-flash-lite</t>
+        </is>
+      </c>
+      <c r="W14" s="2" t="inlineStr">
+        <is>
+          <t>פרומפט מומלץ – טופסי התחשבנות v2</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" s="7" t="n">
+        <v>46292.77593888889</v>
+      </c>
+      <c r="C15" s="4" t="inlineStr">
+        <is>
+          <t>דורש בדיקה</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>• סכום השורות (14,100.00) שונה מהסה"כ לפני מע"מ (12,500.00)
+• סה"כ לפני מע"מ + מע"מ = 14,625.00, אך הסה"כ לתשלום בטופס הוא 15,625.00</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>מייל נכנס</t>
+        </is>
+      </c>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t>גיא כהן &lt;mail4games21@gmail.com&gt;</t>
+        </is>
+      </c>
+      <c r="G15" s="2" t="inlineStr">
+        <is>
+          <t>בדיקת חשבונית (טסט לאוטומציה)</t>
+        </is>
+      </c>
+      <c r="H15" s="2" t="inlineStr">
+        <is>
+          <t>טופס התחשבנות 3 (תקול - אי התאמה בחישוב) - קלין-טק כביסה.pdf</t>
+        </is>
+      </c>
+      <c r="I15" s="2" t="inlineStr">
+        <is>
+          <t>קלין-טק שירותי כביסה וסטריליזציה למוסדות בע"מ</t>
+        </is>
+      </c>
+      <c r="J15" s="2" t="inlineStr">
+        <is>
+          <t>515602119</t>
+        </is>
+      </c>
+      <c r="K15" s="2" t="inlineStr">
+        <is>
+          <t>טופס התחשבנות</t>
+        </is>
+      </c>
+      <c r="L15" s="2" t="inlineStr">
+        <is>
+          <t>CT-2026-409</t>
+        </is>
+      </c>
+      <c r="M15" s="8" t="n">
+        <v>46275</v>
+      </c>
+      <c r="N15" s="8" t="n">
+        <v>46235</v>
+      </c>
+      <c r="O15" s="8" t="n">
+        <v>46265</v>
+      </c>
+      <c r="P15" s="2" t="inlineStr">
+        <is>
+          <t>ILS</t>
+        </is>
+      </c>
+      <c r="Q15" s="6" t="n">
+        <v>12500</v>
+      </c>
+      <c r="R15" s="2" t="n">
+        <v>17</v>
+      </c>
+      <c r="S15" s="6" t="n">
+        <v>2125</v>
+      </c>
+      <c r="T15" s="6" t="n">
+        <v>15625</v>
+      </c>
+      <c r="U15" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="V15" s="2" t="inlineStr">
+        <is>
+          <t>gemini/gemini-3.5-flash-lite</t>
+        </is>
+      </c>
+      <c r="W15" s="2" t="inlineStr">
+        <is>
+          <t>פרומפט מומלץ – טופסי התחשבנות v2</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" s="7" t="n">
+        <v>46292.77600978009</v>
+      </c>
+      <c r="C16" s="4" t="inlineStr">
+        <is>
+          <t>דורש בדיקה</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>• שורה 2: 250 × 16.00 = 4,000.00, אך בטופס מופיע 4,800.00
+• מע"מ 17% על 18,700.00 צריך להיות 3,179.00, אך בטופס מופיע 3,366.00</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>מייל נכנס</t>
+        </is>
+      </c>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t>גיא כהן &lt;mail4games21@gmail.com&gt;</t>
+        </is>
+      </c>
+      <c r="G16" s="2" t="inlineStr">
+        <is>
+          <t>בדיקת חשבונית (טסט לאוטומציה)</t>
+        </is>
+      </c>
+      <c r="H16" s="2" t="inlineStr">
+        <is>
+          <t>טופס התחשבנות 5 (תקול - טעות כפל בשורה ומע_מ שגוי) - שפע קייטרינג.pdf</t>
+        </is>
+      </c>
+      <c r="I16" s="2" t="inlineStr">
+        <is>
+          <t>שפע טעמים - הסעדה וקייטרינג למוסדות רפואיים בע"מ</t>
+        </is>
+      </c>
+      <c r="J16" s="2" t="inlineStr">
+        <is>
+          <t>511209844</t>
+        </is>
+      </c>
+      <c r="K16" s="2" t="inlineStr">
+        <is>
+          <t>חשבונית ריכוז</t>
+        </is>
+      </c>
+      <c r="L16" s="2" t="inlineStr">
+        <is>
+          <t>SH-2026-9912</t>
+        </is>
+      </c>
+      <c r="M16" s="8" t="n">
+        <v>46267</v>
+      </c>
+      <c r="N16" s="8" t="n">
+        <v>46235</v>
+      </c>
+      <c r="O16" s="8" t="n">
+        <v>46265</v>
+      </c>
+      <c r="P16" s="2" t="inlineStr">
+        <is>
+          <t>ILS</t>
+        </is>
+      </c>
+      <c r="Q16" s="6" t="n">
+        <v>18700</v>
+      </c>
+      <c r="R16" s="2" t="n">
+        <v>17</v>
+      </c>
+      <c r="S16" s="6" t="n">
+        <v>3366</v>
+      </c>
+      <c r="T16" s="6" t="n">
+        <v>22066</v>
+      </c>
+      <c r="U16" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="V16" s="2" t="inlineStr">
+        <is>
+          <t>gemini/gemini-3.5-flash-lite</t>
+        </is>
+      </c>
+      <c r="W16" s="2" t="inlineStr">
+        <is>
+          <t>פרומפט מומלץ – טופסי התחשבנות v2</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" s="7" t="n">
+        <v>46292.77607967579</v>
+      </c>
+      <c r="C17" s="9" t="inlineStr">
+        <is>
+          <t>תקין</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr"/>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>מייל נכנס</t>
+        </is>
+      </c>
+      <c r="F17" s="2" t="inlineStr">
+        <is>
+          <t>גיא כהן &lt;mail4games21@gmail.com&gt;</t>
+        </is>
+      </c>
+      <c r="G17" s="2" t="inlineStr">
+        <is>
+          <t>בדיקת חשבונית (טסט לאוטומציה)</t>
+        </is>
+      </c>
+      <c r="H17" s="2" t="inlineStr">
+        <is>
+          <t>טופס התחשבנות ספק - מדי-פארם בע_מ.pdf</t>
+        </is>
+      </c>
+      <c r="I17" s="2" t="inlineStr">
+        <is>
+          <t>מדי-פארם ציוד רפואי וסיעודי בע"מ</t>
+        </is>
+      </c>
+      <c r="J17" s="2" t="inlineStr">
+        <is>
+          <t>514892031</t>
+        </is>
+      </c>
+      <c r="K17" s="2" t="inlineStr">
+        <is>
+          <t>טופס התחשבנות ספק / חשבונית ריכוז</t>
+        </is>
+      </c>
+      <c r="L17" s="2" t="inlineStr">
+        <is>
+          <t>MP-2026-0894</t>
+        </is>
+      </c>
+      <c r="M17" s="8" t="n">
+        <v>46280</v>
+      </c>
+      <c r="N17" s="8" t="n">
+        <v>46235</v>
+      </c>
+      <c r="O17" s="8" t="n">
+        <v>46265</v>
+      </c>
+      <c r="P17" s="2" t="inlineStr">
+        <is>
+          <t>ILS</t>
+        </is>
+      </c>
+      <c r="Q17" s="6" t="n">
+        <v>16000</v>
+      </c>
+      <c r="R17" s="2" t="n">
+        <v>17</v>
+      </c>
+      <c r="S17" s="6" t="n">
+        <v>2720</v>
+      </c>
+      <c r="T17" s="6" t="n">
+        <v>18720</v>
+      </c>
+      <c r="U17" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="V17" s="2" t="inlineStr">
+        <is>
+          <t>gemini/gemini-3.5-flash-lite</t>
+        </is>
+      </c>
+      <c r="W17" s="2" t="inlineStr">
+        <is>
+          <t>פרומפט מומלץ – טופסי התחשבנות v2</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:W7"/>
+  <autoFilter ref="A1:W17"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1155,7 +2038,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J24"/>
+  <dimension ref="A1:J52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -2142,8 +3025,1112 @@
         </is>
       </c>
     </row>
+    <row r="25">
+      <c r="A25" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>קלין-טק שירותי כביסה וסטריליזציה למוסדות בע"מ</t>
+        </is>
+      </c>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t>CT-2026-409</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E25" s="8" t="n">
+        <v>46241</v>
+      </c>
+      <c r="F25" s="2" t="inlineStr">
+        <is>
+          <t>כביסה וחיטוי תרמי של מצעים, סדינים ומגבות (לפי משקל בק"ג)</t>
+        </is>
+      </c>
+      <c r="G25" s="2" t="n">
+        <v>1200</v>
+      </c>
+      <c r="H25" s="6" t="n">
+        <v>6.5</v>
+      </c>
+      <c r="I25" s="6" t="n">
+        <v>7800</v>
+      </c>
+      <c r="J25" s="2" t="inlineStr">
+        <is>
+          <t>תקין</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>קלין-טק שירותי כביסה וסטריליזציה למוסדות בע"מ</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>CT-2026-409</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="E26" s="8" t="n">
+        <v>46249</v>
+      </c>
+      <c r="F26" s="2" t="inlineStr">
+        <is>
+          <t>ניקוי יבש, חיטוי וגיהוץ מדי צוות רפואי וסיעודי (יחידות)</t>
+        </is>
+      </c>
+      <c r="G26" s="2" t="n">
+        <v>150</v>
+      </c>
+      <c r="H26" s="6" t="n">
+        <v>18</v>
+      </c>
+      <c r="I26" s="6" t="n">
+        <v>2700</v>
+      </c>
+      <c r="J26" s="2" t="inlineStr">
+        <is>
+          <t>תקין</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>קלין-טק שירותי כביסה וסטריליזציה למוסדות בע"מ</t>
+        </is>
+      </c>
+      <c r="C27" s="2" t="inlineStr">
+        <is>
+          <t>CT-2026-409</t>
+        </is>
+      </c>
+      <c r="D27" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="E27" s="8" t="n">
+        <v>46257</v>
+      </c>
+      <c r="F27" s="2" t="inlineStr">
+        <is>
+          <t>טיפול מיוחד בכביסה מזוהמת ואריזת ואקום לחדרי בידוד</t>
+        </is>
+      </c>
+      <c r="G27" s="2" t="n">
+        <v>80</v>
+      </c>
+      <c r="H27" s="6" t="n">
+        <v>25</v>
+      </c>
+      <c r="I27" s="6" t="n">
+        <v>2000</v>
+      </c>
+      <c r="J27" s="2" t="inlineStr">
+        <is>
+          <t>תקין</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>קלין-טק שירותי כביסה וסטריליזציה למוסדות בע"מ</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t>CT-2026-409</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="E28" s="8" t="n">
+        <v>46265</v>
+      </c>
+      <c r="F28" s="2" t="inlineStr">
+        <is>
+          <t>דמי הובלה, איסוף והפצה שבועיים במשאית ייעודית (4 סבבים)</t>
+        </is>
+      </c>
+      <c r="G28" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="H28" s="6" t="n">
+        <v>400</v>
+      </c>
+      <c r="I28" s="6" t="n">
+        <v>1600</v>
+      </c>
+      <c r="J28" s="2" t="inlineStr">
+        <is>
+          <t>תקין</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="B29" s="2" t="inlineStr">
+        <is>
+          <t>שפע טעמים - הסעדה וקייטרינג למוסדות רפואיים בע"מ</t>
+        </is>
+      </c>
+      <c r="C29" s="2" t="inlineStr">
+        <is>
+          <t>SH-2026-9912</t>
+        </is>
+      </c>
+      <c r="D29" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E29" s="8" t="n">
+        <v>46244</v>
+      </c>
+      <c r="F29" s="2" t="inlineStr">
+        <is>
+          <t>מנות צהריים חמות מותאמות (דל נתרן / מרקם טחון) - עשרת ראשונה</t>
+        </is>
+      </c>
+      <c r="G29" s="2" t="n">
+        <v>400</v>
+      </c>
+      <c r="H29" s="6" t="n">
+        <v>28</v>
+      </c>
+      <c r="I29" s="6" t="n">
+        <v>11200</v>
+      </c>
+      <c r="J29" s="2" t="inlineStr">
+        <is>
+          <t>תקין</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t>שפע טעמים - הסעדה וקייטרינג למוסדות רפואיים בע"מ</t>
+        </is>
+      </c>
+      <c r="C30" s="2" t="inlineStr">
+        <is>
+          <t>SH-2026-9912</t>
+        </is>
+      </c>
+      <c r="D30" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="E30" s="8" t="n">
+        <v>46254</v>
+      </c>
+      <c r="F30" s="2" t="inlineStr">
+        <is>
+          <t>מארזי ארוחות בוקר וערב אישיים למחלקת שיקום ותשושי נפש</t>
+        </is>
+      </c>
+      <c r="G30" s="2" t="n">
+        <v>250</v>
+      </c>
+      <c r="H30" s="6" t="n">
+        <v>16</v>
+      </c>
+      <c r="I30" s="6" t="n">
+        <v>4800</v>
+      </c>
+      <c r="J30" s="2" t="inlineStr">
+        <is>
+          <t>שגיאת חישוב</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="B31" s="2" t="inlineStr">
+        <is>
+          <t>שפע טעמים - הסעדה וקייטרינג למוסדות רפואיים בע"מ</t>
+        </is>
+      </c>
+      <c r="C31" s="2" t="inlineStr">
+        <is>
+          <t>SH-2026-9912</t>
+        </is>
+      </c>
+      <c r="D31" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="E31" s="8" t="n">
+        <v>46265</v>
+      </c>
+      <c r="F31" s="2" t="inlineStr">
+        <is>
+          <t>אספקת פורמולות העשרה תזונתית ואבקות חלבון קליניות</t>
+        </is>
+      </c>
+      <c r="G31" s="2" t="n">
+        <v>60</v>
+      </c>
+      <c r="H31" s="6" t="n">
+        <v>45</v>
+      </c>
+      <c r="I31" s="6" t="n">
+        <v>2700</v>
+      </c>
+      <c r="J31" s="2" t="inlineStr">
+        <is>
+          <t>תקין</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="n">
+        <v>11</v>
+      </c>
+      <c r="B32" s="2" t="inlineStr">
+        <is>
+          <t>מדי-פארם ציוד רפואי וסיעודי בע"מ</t>
+        </is>
+      </c>
+      <c r="C32" s="2" t="inlineStr">
+        <is>
+          <t>MP-2026-0894</t>
+        </is>
+      </c>
+      <c r="D32" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E32" s="8" t="n">
+        <v>46238</v>
+      </c>
+      <c r="F32" s="2" t="inlineStr">
+        <is>
+          <t>ערכות ציוד סיעודי מתכלה – אספקה חודשית מרוכזת תעודת משלוח מס' 88412 | חלוקה למחלקות א'–ג'</t>
+        </is>
+      </c>
+      <c r="G32" s="2" t="n">
+        <v>25</v>
+      </c>
+      <c r="H32" s="6" t="n">
+        <v>320</v>
+      </c>
+      <c r="I32" s="6" t="n">
+        <v>8000</v>
+      </c>
+      <c r="J32" s="2" t="inlineStr">
+        <is>
+          <t>תקין</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="n">
+        <v>11</v>
+      </c>
+      <c r="B33" s="2" t="inlineStr">
+        <is>
+          <t>מדי-פארם ציוד רפואי וסיעודי בע"מ</t>
+        </is>
+      </c>
+      <c r="C33" s="2" t="inlineStr">
+        <is>
+          <t>MP-2026-0894</t>
+        </is>
+      </c>
+      <c r="D33" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="E33" s="8" t="n">
+        <v>46246</v>
+      </c>
+      <c r="F33" s="2" t="inlineStr">
+        <is>
+          <t>תחזוקה תקופתית וכיול מכשירי ניטור ומדדי לחץ דם קריאת שירות מרוכזת מס' 4190 | כולל הנפקת תעודות תקינות</t>
+        </is>
+      </c>
+      <c r="G33" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="H33" s="6" t="n">
+        <v>250</v>
+      </c>
+      <c r="I33" s="6" t="n">
+        <v>3000</v>
+      </c>
+      <c r="J33" s="2" t="inlineStr">
+        <is>
+          <t>תקין</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="n">
+        <v>11</v>
+      </c>
+      <c r="B34" s="2" t="inlineStr">
+        <is>
+          <t>מדי-פארם ציוד רפואי וסיעודי בע"מ</t>
+        </is>
+      </c>
+      <c r="C34" s="2" t="inlineStr">
+        <is>
+          <t>MP-2026-0894</t>
+        </is>
+      </c>
+      <c r="D34" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="E34" s="8" t="n">
+        <v>46254</v>
+      </c>
+      <c r="F34" s="2" t="inlineStr">
+        <is>
+          <t>השכרת מיטות סיעודיות חשמליות ומזרני לחץ דינמיים חיוב שכירות חודשי קבוע עבור חודש אוגוסט 2026</t>
+        </is>
+      </c>
+      <c r="G34" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="H34" s="6" t="n">
+        <v>450</v>
+      </c>
+      <c r="I34" s="6" t="n">
+        <v>3600</v>
+      </c>
+      <c r="J34" s="2" t="inlineStr">
+        <is>
+          <t>תקין</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="n">
+        <v>11</v>
+      </c>
+      <c r="B35" s="2" t="inlineStr">
+        <is>
+          <t>מדי-פארם ציוד רפואי וסיעודי בע"מ</t>
+        </is>
+      </c>
+      <c r="C35" s="2" t="inlineStr">
+        <is>
+          <t>MP-2026-0894</t>
+        </is>
+      </c>
+      <c r="D35" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="E35" s="8" t="n">
+        <v>46262</v>
+      </c>
+      <c r="F35" s="2" t="inlineStr">
+        <is>
+          <t>מילוי ואספקה דחופה של מחוללי ובלוני חמצן ניידים תעודת משלוח מס' 88905 | כולל בדיקת וסתים בטיחותית</t>
+        </is>
+      </c>
+      <c r="G35" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="H35" s="6" t="n">
+        <v>280</v>
+      </c>
+      <c r="I35" s="6" t="n">
+        <v>1400</v>
+      </c>
+      <c r="J35" s="2" t="inlineStr">
+        <is>
+          <t>תקין</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="B36" s="2" t="inlineStr">
+        <is>
+          <t>א.ב. הנדסת מיזוג אוויר ואחזקת מבנים</t>
+        </is>
+      </c>
+      <c r="C36" s="2" t="n"/>
+      <c r="D36" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E36" s="8" t="n">
+        <v>46237</v>
+      </c>
+      <c r="F36" s="2" t="inlineStr">
+        <is>
+          <t>החלפת מדחס מרכזי במערכת צ'ילר ראשית כולל פירוק והרכבה</t>
+        </is>
+      </c>
+      <c r="G36" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="H36" s="6" t="n">
+        <v>6400</v>
+      </c>
+      <c r="I36" s="6" t="n">
+        <v>6400</v>
+      </c>
+      <c r="J36" s="2" t="inlineStr">
+        <is>
+          <t>תקין</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="B37" s="2" t="inlineStr">
+        <is>
+          <t>א.ב. הנדסת מיזוג אוויר ואחזקת מבנים</t>
+        </is>
+      </c>
+      <c r="C37" s="2" t="n"/>
+      <c r="D37" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="E37" s="8" t="n">
+        <v>46245</v>
+      </c>
+      <c r="F37" s="2" t="inlineStr">
+        <is>
+          <t>ניקוי סוללות, שטיפת פילטרים וחיטוי תעלות ב35- חדרי אשפוז</t>
+        </is>
+      </c>
+      <c r="G37" s="2" t="n">
+        <v>35</v>
+      </c>
+      <c r="H37" s="6" t="n">
+        <v>90</v>
+      </c>
+      <c r="I37" s="6" t="n">
+        <v>3150</v>
+      </c>
+      <c r="J37" s="2" t="inlineStr">
+        <is>
+          <t>תקין</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="B38" s="2" t="inlineStr">
+        <is>
+          <t>א.ב. הנדסת מיזוג אוויר ואחזקת מבנים</t>
+        </is>
+      </c>
+      <c r="C38" s="2" t="n"/>
+      <c r="D38" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="E38" s="8" t="n">
+        <v>46260</v>
+      </c>
+      <c r="F38" s="2" t="inlineStr">
+        <is>
+          <t>איתור דליפת גז בצנרת גג ומילוי גז פריאון A410R( לפי משקל)</t>
+        </is>
+      </c>
+      <c r="G38" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="H38" s="6" t="n"/>
+      <c r="I38" s="6" t="n"/>
+      <c r="J38" s="2" t="inlineStr">
+        <is>
+          <t>חסר סכום</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="2" t="n">
+        <v>13</v>
+      </c>
+      <c r="B39" s="2" t="inlineStr">
+        <is>
+          <t>ש.ל.ה שירותי לוגיסטיקה והסעות רפואיות בע"מ</t>
+        </is>
+      </c>
+      <c r="C39" s="2" t="inlineStr">
+        <is>
+          <t>SLH-88421</t>
+        </is>
+      </c>
+      <c r="D39" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E39" s="8" t="n">
+        <v>46239</v>
+      </c>
+      <c r="F39" s="2" t="inlineStr">
+        <is>
+          <t>הסעת מטופלים בכיסאות גלגלים (אמבולנס מותאם) קו מרכז גריאטרי גולדנקייר ← מרפאות חוץ שיבא תל השומר</t>
+        </is>
+      </c>
+      <c r="G39" s="2" t="n">
+        <v>18</v>
+      </c>
+      <c r="H39" s="6" t="n">
+        <v>350</v>
+      </c>
+      <c r="I39" s="6" t="n">
+        <v>6300</v>
+      </c>
+      <c r="J39" s="2" t="inlineStr">
+        <is>
+          <t>תקין</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="2" t="n">
+        <v>13</v>
+      </c>
+      <c r="B40" s="2" t="inlineStr">
+        <is>
+          <t>ש.ל.ה שירותי לוגיסטיקה והסעות רפואיות בע"מ</t>
+        </is>
+      </c>
+      <c r="C40" s="2" t="inlineStr">
+        <is>
+          <t>SLH-88421</t>
+        </is>
+      </c>
+      <c r="D40" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="E40" s="8" t="n">
+        <v>46248</v>
+      </c>
+      <c r="F40" s="2" t="inlineStr">
+        <is>
+          <t>שינוע דגימות מעבדה וציוד סטרילי בקירור (2–8 מעלות) איסוף יומי מרוכז מכלל מחלקות האשפוז והעברה למעבדה מרכזית</t>
+        </is>
+      </c>
+      <c r="G40" s="2" t="n">
+        <v>22</v>
+      </c>
+      <c r="H40" s="6" t="n">
+        <v>150</v>
+      </c>
+      <c r="I40" s="6" t="n">
+        <v>3300</v>
+      </c>
+      <c r="J40" s="2" t="inlineStr">
+        <is>
+          <t>תקין</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="2" t="n">
+        <v>13</v>
+      </c>
+      <c r="B41" s="2" t="inlineStr">
+        <is>
+          <t>ש.ל.ה שירותי לוגיסטיקה והסעות רפואיות בע"מ</t>
+        </is>
+      </c>
+      <c r="C41" s="2" t="inlineStr">
+        <is>
+          <t>SLH-88421</t>
+        </is>
+      </c>
+      <c r="D41" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="E41" s="8" t="n">
+        <v>46259</v>
+      </c>
+      <c r="F41" s="2" t="inlineStr">
+        <is>
+          <t>הזנקת חירום לילית – פינוי מטופל בליווי חובש כולל תוספת תעריף לילה והמתנת צוות רפואי בחדר מיון איכילוב</t>
+        </is>
+      </c>
+      <c r="G41" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="H41" s="6" t="n">
+        <v>700</v>
+      </c>
+      <c r="I41" s="6" t="n">
+        <v>1400</v>
+      </c>
+      <c r="J41" s="2" t="inlineStr">
+        <is>
+          <t>תקין</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="2" t="n">
+        <v>14</v>
+      </c>
+      <c r="B42" s="2" t="inlineStr">
+        <is>
+          <t>קלין-טק שירותי כביסה וסטריליזציה למוסדות בע"מ</t>
+        </is>
+      </c>
+      <c r="C42" s="2" t="inlineStr">
+        <is>
+          <t>CT-2026-409</t>
+        </is>
+      </c>
+      <c r="D42" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E42" s="8" t="n">
+        <v>46241</v>
+      </c>
+      <c r="F42" s="2" t="inlineStr">
+        <is>
+          <t>כביסה וחיטוי תרמי של מצעים, סדינים ומגבות (לפי משקל בק"ג)</t>
+        </is>
+      </c>
+      <c r="G42" s="2" t="n">
+        <v>1200</v>
+      </c>
+      <c r="H42" s="6" t="n">
+        <v>6.5</v>
+      </c>
+      <c r="I42" s="6" t="n">
+        <v>7800</v>
+      </c>
+      <c r="J42" s="2" t="inlineStr">
+        <is>
+          <t>תקין</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="2" t="n">
+        <v>14</v>
+      </c>
+      <c r="B43" s="2" t="inlineStr">
+        <is>
+          <t>קלין-טק שירותי כביסה וסטריליזציה למוסדות בע"מ</t>
+        </is>
+      </c>
+      <c r="C43" s="2" t="inlineStr">
+        <is>
+          <t>CT-2026-409</t>
+        </is>
+      </c>
+      <c r="D43" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="E43" s="8" t="n">
+        <v>46249</v>
+      </c>
+      <c r="F43" s="2" t="inlineStr">
+        <is>
+          <t>ניקוי יבש, חיטוי וגיהוץ מדי צוות רפואי וסיעודי (יחידות)</t>
+        </is>
+      </c>
+      <c r="G43" s="2" t="n">
+        <v>150</v>
+      </c>
+      <c r="H43" s="6" t="n">
+        <v>18</v>
+      </c>
+      <c r="I43" s="6" t="n">
+        <v>2700</v>
+      </c>
+      <c r="J43" s="2" t="inlineStr">
+        <is>
+          <t>תקין</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="2" t="n">
+        <v>14</v>
+      </c>
+      <c r="B44" s="2" t="inlineStr">
+        <is>
+          <t>קלין-טק שירותי כביסה וסטריליזציה למוסדות בע"מ</t>
+        </is>
+      </c>
+      <c r="C44" s="2" t="inlineStr">
+        <is>
+          <t>CT-2026-409</t>
+        </is>
+      </c>
+      <c r="D44" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="E44" s="8" t="n">
+        <v>46257</v>
+      </c>
+      <c r="F44" s="2" t="inlineStr">
+        <is>
+          <t>טיפול מיוחד בכביסה מזוהמת ואריזת ואקום לחדרי בידוד</t>
+        </is>
+      </c>
+      <c r="G44" s="2" t="n">
+        <v>80</v>
+      </c>
+      <c r="H44" s="6" t="n">
+        <v>25</v>
+      </c>
+      <c r="I44" s="6" t="n">
+        <v>2000</v>
+      </c>
+      <c r="J44" s="2" t="inlineStr">
+        <is>
+          <t>תקין</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="2" t="n">
+        <v>14</v>
+      </c>
+      <c r="B45" s="2" t="inlineStr">
+        <is>
+          <t>קלין-טק שירותי כביסה וסטריליזציה למוסדות בע"מ</t>
+        </is>
+      </c>
+      <c r="C45" s="2" t="inlineStr">
+        <is>
+          <t>CT-2026-409</t>
+        </is>
+      </c>
+      <c r="D45" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="E45" s="8" t="n">
+        <v>46265</v>
+      </c>
+      <c r="F45" s="2" t="inlineStr">
+        <is>
+          <t>דמי הובלה, איסוף והפצה שבועיים במשאית ייעודית (4 סבבים)</t>
+        </is>
+      </c>
+      <c r="G45" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="H45" s="6" t="n">
+        <v>400</v>
+      </c>
+      <c r="I45" s="6" t="n">
+        <v>1600</v>
+      </c>
+      <c r="J45" s="2" t="inlineStr">
+        <is>
+          <t>תקין</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="B46" s="2" t="inlineStr">
+        <is>
+          <t>שפע טעמים - הסעדה וקייטרינג למוסדות רפואיים בע"מ</t>
+        </is>
+      </c>
+      <c r="C46" s="2" t="inlineStr">
+        <is>
+          <t>SH-2026-9912</t>
+        </is>
+      </c>
+      <c r="D46" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E46" s="8" t="n">
+        <v>46244</v>
+      </c>
+      <c r="F46" s="2" t="inlineStr">
+        <is>
+          <t>מנות צהריים חמות מותאמות (דל נתרן / מרקם טחון) – עשרת ראשונה</t>
+        </is>
+      </c>
+      <c r="G46" s="2" t="n">
+        <v>400</v>
+      </c>
+      <c r="H46" s="6" t="n">
+        <v>28</v>
+      </c>
+      <c r="I46" s="6" t="n">
+        <v>11200</v>
+      </c>
+      <c r="J46" s="2" t="inlineStr">
+        <is>
+          <t>תקין</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="B47" s="2" t="inlineStr">
+        <is>
+          <t>שפע טעמים - הסעדה וקייטרינג למוסדות רפואיים בע"מ</t>
+        </is>
+      </c>
+      <c r="C47" s="2" t="inlineStr">
+        <is>
+          <t>SH-2026-9912</t>
+        </is>
+      </c>
+      <c r="D47" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="E47" s="8" t="n">
+        <v>46254</v>
+      </c>
+      <c r="F47" s="2" t="inlineStr">
+        <is>
+          <t>מארזי ארוחות בוקר וערב אישיים למחלקת שיקום ותשושי נפש</t>
+        </is>
+      </c>
+      <c r="G47" s="2" t="n">
+        <v>250</v>
+      </c>
+      <c r="H47" s="6" t="n">
+        <v>16</v>
+      </c>
+      <c r="I47" s="6" t="n">
+        <v>4800</v>
+      </c>
+      <c r="J47" s="2" t="inlineStr">
+        <is>
+          <t>שגיאת חישוב</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="B48" s="2" t="inlineStr">
+        <is>
+          <t>שפע טעמים - הסעדה וקייטרינג למוסדות רפואיים בע"מ</t>
+        </is>
+      </c>
+      <c r="C48" s="2" t="inlineStr">
+        <is>
+          <t>SH-2026-9912</t>
+        </is>
+      </c>
+      <c r="D48" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="E48" s="8" t="n">
+        <v>46265</v>
+      </c>
+      <c r="F48" s="2" t="inlineStr">
+        <is>
+          <t>אספקת פורמולות העשרה תזונתית ואבקות חלבון קליניות</t>
+        </is>
+      </c>
+      <c r="G48" s="2" t="n">
+        <v>60</v>
+      </c>
+      <c r="H48" s="6" t="n">
+        <v>45</v>
+      </c>
+      <c r="I48" s="6" t="n">
+        <v>2700</v>
+      </c>
+      <c r="J48" s="2" t="inlineStr">
+        <is>
+          <t>תקין</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="2" t="n">
+        <v>16</v>
+      </c>
+      <c r="B49" s="2" t="inlineStr">
+        <is>
+          <t>מדי-פארם ציוד רפואי וסיעודי בע"מ</t>
+        </is>
+      </c>
+      <c r="C49" s="2" t="inlineStr">
+        <is>
+          <t>MP-2026-0894</t>
+        </is>
+      </c>
+      <c r="D49" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E49" s="8" t="n">
+        <v>46238</v>
+      </c>
+      <c r="F49" s="2" t="inlineStr">
+        <is>
+          <t>ערכות ציוד סיעודי מתכלה – אספקה חודשית מרוכזת תעודת משלוח מס' 88412 | חלוקה למחלקות א'–ג'</t>
+        </is>
+      </c>
+      <c r="G49" s="2" t="n">
+        <v>25</v>
+      </c>
+      <c r="H49" s="6" t="n">
+        <v>320</v>
+      </c>
+      <c r="I49" s="6" t="n">
+        <v>8000</v>
+      </c>
+      <c r="J49" s="2" t="inlineStr">
+        <is>
+          <t>תקין</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="2" t="n">
+        <v>16</v>
+      </c>
+      <c r="B50" s="2" t="inlineStr">
+        <is>
+          <t>מדי-פארם ציוד רפואי וסיעודי בע"מ</t>
+        </is>
+      </c>
+      <c r="C50" s="2" t="inlineStr">
+        <is>
+          <t>MP-2026-0894</t>
+        </is>
+      </c>
+      <c r="D50" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="E50" s="8" t="n">
+        <v>46246</v>
+      </c>
+      <c r="F50" s="2" t="inlineStr">
+        <is>
+          <t>תחזוקה תקופתית וכיול מכשירי ניטור ומדדי לחץ דם קריאת שירות מרוכזת מס' 4190 | כולל הנפקת תעודות תקינות</t>
+        </is>
+      </c>
+      <c r="G50" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="H50" s="6" t="n">
+        <v>250</v>
+      </c>
+      <c r="I50" s="6" t="n">
+        <v>3000</v>
+      </c>
+      <c r="J50" s="2" t="inlineStr">
+        <is>
+          <t>תקין</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="2" t="n">
+        <v>16</v>
+      </c>
+      <c r="B51" s="2" t="inlineStr">
+        <is>
+          <t>מדי-פארם ציוד רפואי וסיעודי בע"מ</t>
+        </is>
+      </c>
+      <c r="C51" s="2" t="inlineStr">
+        <is>
+          <t>MP-2026-0894</t>
+        </is>
+      </c>
+      <c r="D51" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="E51" s="8" t="n">
+        <v>46254</v>
+      </c>
+      <c r="F51" s="2" t="inlineStr">
+        <is>
+          <t>השכרת מיטות סיעודיות חשמליות ומזרני לחץ דינמיים חיוב שכירות חודשי קבוע עבור חודש אוגוסט 2026</t>
+        </is>
+      </c>
+      <c r="G51" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="H51" s="6" t="n">
+        <v>450</v>
+      </c>
+      <c r="I51" s="6" t="n">
+        <v>3600</v>
+      </c>
+      <c r="J51" s="2" t="inlineStr">
+        <is>
+          <t>תקין</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="2" t="n">
+        <v>16</v>
+      </c>
+      <c r="B52" s="2" t="inlineStr">
+        <is>
+          <t>מדי-פארם ציוד רפואי וסיעודי בע"מ</t>
+        </is>
+      </c>
+      <c r="C52" s="2" t="inlineStr">
+        <is>
+          <t>MP-2026-0894</t>
+        </is>
+      </c>
+      <c r="D52" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="E52" s="8" t="n">
+        <v>46262</v>
+      </c>
+      <c r="F52" s="2" t="inlineStr">
+        <is>
+          <t>מילוי ואספקה דחופה של מחוללי ובלוני חמצן ניידים תעודת משלוח מס' 88905 | כולל בדיקת וסתים בטיחותית</t>
+        </is>
+      </c>
+      <c r="G52" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="H52" s="6" t="n">
+        <v>280</v>
+      </c>
+      <c r="I52" s="6" t="n">
+        <v>1400</v>
+      </c>
+      <c r="J52" s="2" t="inlineStr">
+        <is>
+          <t>תקין</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J24"/>
+  <autoFilter ref="A1:J52"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: add document labeling and regression testing suite with frontend UI and backend services
</commit_message>
<xml_diff>
--- a/data/GoldenCare_Master.xlsx
+++ b/data/GoldenCare_Master.xlsx
@@ -10,7 +10,7 @@
     <sheet name="שורות חיוב" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'מסמכים'!$A$1:$W$9</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'מסמכים'!$A$1:$W$29</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'שורות חיוב'!$A$1:$J$95</definedName>
   </definedNames>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -19,11 +19,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="4">
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="DD/MM/YYYY HH:MM"/>
     <numFmt numFmtId="165" formatCode="DD/MM/YYYY"/>
     <numFmt numFmtId="166" formatCode="yyyy-mm-dd h:mm:ss"/>
-    <numFmt numFmtId="167" formatCode="yyyy-mm-dd"/>
   </numFmts>
   <fonts count="2">
     <font>
@@ -40,7 +39,7 @@
       <sz val="11"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
@@ -67,6 +66,11 @@
         <fgColor rgb="00C6EFCE"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFC7CE"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -80,7 +84,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -116,6 +120,9 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -483,7 +490,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:W9"/>
+  <dimension ref="A1:W29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -1269,7 +1276,7 @@
         <v>29</v>
       </c>
       <c r="B9" s="11" t="n">
-        <v>46292.82578534211</v>
+        <v>46292.82578534722</v>
       </c>
       <c r="C9" s="9" t="inlineStr">
         <is>
@@ -1349,8 +1356,1180 @@
         </is>
       </c>
     </row>
+    <row r="10">
+      <c r="A10" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="B10" s="11" t="n">
+        <v>46293.6548978588</v>
+      </c>
+      <c r="C10" s="13" t="inlineStr">
+        <is>
+          <t>חילוץ נכשל</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>חריגה ממכסת ה-API של ספק ה-AI. פרטים: gemini/gemini-3.8-flash: 429 You exceeded your current quota, please check your plan and billing details. For more information on this error, head to: https://ai.goo | gemini/gemini-3.7-flash: 429 You exceeded your current quota, please check your plan and billing details. For more information on this error, head to: https://ai.goo | gemini/gemini-3.5-flash: 429 You exceeded your current quota, please check your plan and billing details. For more information on this error, head to: https://ai.goo | gemini/gemini-3.5-flash-lite: 504 Deadline expired before operation could complete.</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>מייל נכנס</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>גיא כהן &lt;mail4games21@gmail.com&gt;</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>בדיקת חשבונית (טסט לאוטומציה)</t>
+        </is>
+      </c>
+      <c r="H10" s="2" t="inlineStr">
+        <is>
+          <t>טופס התחשבנות 4 (תקול - חוסר שדות וערכים לא מספריים) - א.ב. מיזוג.pdf</t>
+        </is>
+      </c>
+      <c r="I10" s="2" t="n"/>
+      <c r="J10" s="2" t="n"/>
+      <c r="K10" s="2" t="n"/>
+      <c r="L10" s="2" t="n"/>
+      <c r="M10" s="12" t="n"/>
+      <c r="N10" s="12" t="n"/>
+      <c r="O10" s="12" t="n"/>
+      <c r="P10" s="2" t="n"/>
+      <c r="Q10" s="5" t="n"/>
+      <c r="R10" s="2" t="n"/>
+      <c r="S10" s="5" t="n"/>
+      <c r="T10" s="5" t="n"/>
+      <c r="U10" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="V10" s="2" t="n"/>
+      <c r="W10" s="2" t="inlineStr">
+        <is>
+          <t>הספק הוא תמיד א ב טכנלוגיות וניסויים (פרומפט תקול)</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="n">
+        <v>31</v>
+      </c>
+      <c r="B11" s="11" t="n">
+        <v>46293.65672305555</v>
+      </c>
+      <c r="C11" s="13" t="inlineStr">
+        <is>
+          <t>חילוץ נכשל</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>חריגה ממכסת ה-API של ספק ה-AI. פרטים: gemini/gemini-3.8-flash: 429 You exceeded your current quota, please check your plan and billing details. For more information on this error, head to: https://ai.goo | gemini/gemini-3.7-flash: 429 You exceeded your current quota, please check your plan and billing details. For more information on this error, head to: https://ai.goo | gemini/gemini-3.5-flash: 429 You exceeded your current quota, please check your plan and billing details. For more information on this error, head to: https://ai.goo | gemini/gemini-3.5-flash-lite: 504 Deadline expired before operation could complete.</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>מייל נכנס</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>גיא כהן &lt;mail4games21@gmail.com&gt;</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>בדיקת חשבונית (טסט לאוטומציה)</t>
+        </is>
+      </c>
+      <c r="H11" s="2" t="inlineStr">
+        <is>
+          <t>טופס התחשבנות 2 (תקין - עיצוב שונה) - ש.ל.ה הסעות רפואיות.pdf</t>
+        </is>
+      </c>
+      <c r="I11" s="2" t="n"/>
+      <c r="J11" s="2" t="n"/>
+      <c r="K11" s="2" t="n"/>
+      <c r="L11" s="2" t="n"/>
+      <c r="M11" s="12" t="n"/>
+      <c r="N11" s="12" t="n"/>
+      <c r="O11" s="12" t="n"/>
+      <c r="P11" s="2" t="n"/>
+      <c r="Q11" s="5" t="n"/>
+      <c r="R11" s="2" t="n"/>
+      <c r="S11" s="5" t="n"/>
+      <c r="T11" s="5" t="n"/>
+      <c r="U11" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="V11" s="2" t="n"/>
+      <c r="W11" s="2" t="inlineStr">
+        <is>
+          <t>הספק הוא תמיד א ב טכנלוגיות וניסויים (פרומפט תקול)</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="n">
+        <v>32</v>
+      </c>
+      <c r="B12" s="11" t="n">
+        <v>46293.6583265625</v>
+      </c>
+      <c r="C12" s="13" t="inlineStr">
+        <is>
+          <t>חילוץ נכשל</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>חריגה ממכסת ה-API של ספק ה-AI. פרטים: gemini/gemini-3.8-flash: 429 You exceeded your current quota, please check your plan and billing details. For more information on this error, head to: https://ai.goo | gemini/gemini-3.7-flash: 429 You exceeded your current quota, please check your plan and billing details. For more information on this error, head to: https://ai.goo | gemini/gemini-3.5-flash: 429 You exceeded your current quota, please check your plan and billing details. For more information on this error, head to: https://ai.goo | gemini/gemini-3.5-flash-lite: 504 Deadline expired before operation could complete.</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>מייל נכנס</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>גיא כהן &lt;mail4games21@gmail.com&gt;</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>בדיקת חשבונית (טסט לאוטומציה)</t>
+        </is>
+      </c>
+      <c r="H12" s="2" t="inlineStr">
+        <is>
+          <t>טופס התחשבנות 3 (תקול - אי התאמה בחישוב) - קלין-טק כביסה.pdf</t>
+        </is>
+      </c>
+      <c r="I12" s="2" t="n"/>
+      <c r="J12" s="2" t="n"/>
+      <c r="K12" s="2" t="n"/>
+      <c r="L12" s="2" t="n"/>
+      <c r="M12" s="12" t="n"/>
+      <c r="N12" s="12" t="n"/>
+      <c r="O12" s="12" t="n"/>
+      <c r="P12" s="2" t="n"/>
+      <c r="Q12" s="5" t="n"/>
+      <c r="R12" s="2" t="n"/>
+      <c r="S12" s="5" t="n"/>
+      <c r="T12" s="5" t="n"/>
+      <c r="U12" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="V12" s="2" t="n"/>
+      <c r="W12" s="2" t="inlineStr">
+        <is>
+          <t>הספק הוא תמיד א ב טכנלוגיות וניסויים (פרומפט תקול)</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="n">
+        <v>33</v>
+      </c>
+      <c r="B13" s="11" t="n">
+        <v>46293.6596515625</v>
+      </c>
+      <c r="C13" s="13" t="inlineStr">
+        <is>
+          <t>חילוץ נכשל</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>חריגה ממכסת ה-API של ספק ה-AI. פרטים: gemini/gemini-3.8-flash: 429 You exceeded your current quota, please check your plan and billing details. For more information on this error, head to: https://ai.goo | gemini/gemini-3.7-flash: 429 You exceeded your current quota, please check your plan and billing details. For more information on this error, head to: https://ai.goo | gemini/gemini-3.5-flash: 429 You exceeded your current quota, please check your plan and billing details. For more information on this error, head to: https://ai.goo | gemini/gemini-3.5-flash-lite: 504 Deadline Exceeded</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>מייל נכנס</t>
+        </is>
+      </c>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>גיא כהן &lt;mail4games21@gmail.com&gt;</t>
+        </is>
+      </c>
+      <c r="G13" s="2" t="inlineStr">
+        <is>
+          <t>בדיקת חשבונית (טסט לאוטומציה)</t>
+        </is>
+      </c>
+      <c r="H13" s="2" t="inlineStr">
+        <is>
+          <t>טופס התחשבנות 5 (תקול - טעות כפל בשורה ומע_מ שגוי) - שפע קייטרינג.pdf</t>
+        </is>
+      </c>
+      <c r="I13" s="2" t="n"/>
+      <c r="J13" s="2" t="n"/>
+      <c r="K13" s="2" t="n"/>
+      <c r="L13" s="2" t="n"/>
+      <c r="M13" s="12" t="n"/>
+      <c r="N13" s="12" t="n"/>
+      <c r="O13" s="12" t="n"/>
+      <c r="P13" s="2" t="n"/>
+      <c r="Q13" s="5" t="n"/>
+      <c r="R13" s="2" t="n"/>
+      <c r="S13" s="5" t="n"/>
+      <c r="T13" s="5" t="n"/>
+      <c r="U13" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="V13" s="2" t="n"/>
+      <c r="W13" s="2" t="inlineStr">
+        <is>
+          <t>הספק הוא תמיד א ב טכנלוגיות וניסויים (פרומפט תקול)</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="n">
+        <v>34</v>
+      </c>
+      <c r="B14" s="11" t="n">
+        <v>46293.66595083333</v>
+      </c>
+      <c r="C14" s="13" t="inlineStr">
+        <is>
+          <t>חילוץ נכשל</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>חריגה ממכסת ה-API של ספק ה-AI. פרטים: gemini/gemini-3.8-flash: 429 You exceeded your current quota, please check your plan and billing details. For more information on this error, head to: https://ai.goo | gemini/gemini-3.7-flash: 429 You exceeded your current quota, please check your plan and billing details. For more information on this error, head to: https://ai.goo | gemini/gemini-3.5-flash: 429 You exceeded your current quota, please check your plan and billing details. For more information on this error, head to: https://ai.goo | gemini/gemini-3.5-flash-lite: Timeout of 60.0s exceeded, last exception: 503 This model is currently experiencing high demand. Spikes in demand are usually temporary. Ple</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>מייל נכנס</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>גיא כהן &lt;mail4games21@gmail.com&gt;</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t>בדיקת חשבונית (טסט לאוטומציה)</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="inlineStr">
+        <is>
+          <t>טופס התחשבנות 4 (תקול - חוסר שדות וערכים לא מספריים) - א.ב. מיזוג.pdf</t>
+        </is>
+      </c>
+      <c r="I14" s="2" t="n"/>
+      <c r="J14" s="2" t="n"/>
+      <c r="K14" s="2" t="n"/>
+      <c r="L14" s="2" t="n"/>
+      <c r="M14" s="12" t="n"/>
+      <c r="N14" s="12" t="n"/>
+      <c r="O14" s="12" t="n"/>
+      <c r="P14" s="2" t="n"/>
+      <c r="Q14" s="5" t="n"/>
+      <c r="R14" s="2" t="n"/>
+      <c r="S14" s="5" t="n"/>
+      <c r="T14" s="5" t="n"/>
+      <c r="U14" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="V14" s="2" t="n"/>
+      <c r="W14" s="2" t="inlineStr">
+        <is>
+          <t>הספק הוא תמיד א ב טכנלוגיות וניסויים (פרומפט תקול)</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="n">
+        <v>35</v>
+      </c>
+      <c r="B15" s="11" t="n">
+        <v>46293.66663254629</v>
+      </c>
+      <c r="C15" s="13" t="inlineStr">
+        <is>
+          <t>חילוץ נכשל</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>חריגה ממכסת ה-API של ספק ה-AI. פרטים: gemini/gemini-3.8-flash: 429 You exceeded your current quota, please check your plan and billing details. For more information on this error, head to: https://ai.goo | gemini/gemini-3.7-flash: 429 You exceeded your current quota, please check your plan and billing details. For more information on this error, head to: https://ai.goo | gemini/gemini-3.5-flash: 429 You exceeded your current quota, please check your plan and billing details. For more information on this error, head to: https://ai.goo | gemini/gemini-3.5-flash-lite: Timeout of 60.0s exceeded, last exception: 503 This model is currently experiencing high demand. Spikes in demand are usually temporary. Ple</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>מייל נכנס</t>
+        </is>
+      </c>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t>גיא כהן &lt;mail4games21@gmail.com&gt;</t>
+        </is>
+      </c>
+      <c r="G15" s="2" t="inlineStr">
+        <is>
+          <t>בדיקת חשבונית (טסט לאוטומציה)</t>
+        </is>
+      </c>
+      <c r="H15" s="2" t="inlineStr">
+        <is>
+          <t>טופס התחשבנות 2 (תקין - עיצוב שונה) - ש.ל.ה הסעות רפואיות.pdf</t>
+        </is>
+      </c>
+      <c r="I15" s="2" t="n"/>
+      <c r="J15" s="2" t="n"/>
+      <c r="K15" s="2" t="n"/>
+      <c r="L15" s="2" t="n"/>
+      <c r="M15" s="12" t="n"/>
+      <c r="N15" s="12" t="n"/>
+      <c r="O15" s="12" t="n"/>
+      <c r="P15" s="2" t="n"/>
+      <c r="Q15" s="5" t="n"/>
+      <c r="R15" s="2" t="n"/>
+      <c r="S15" s="5" t="n"/>
+      <c r="T15" s="5" t="n"/>
+      <c r="U15" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="V15" s="2" t="n"/>
+      <c r="W15" s="2" t="inlineStr">
+        <is>
+          <t>הספק הוא תמיד א ב טכנלוגיות וניסויים (פרומפט תקול)</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="n">
+        <v>36</v>
+      </c>
+      <c r="B16" s="11" t="n">
+        <v>46293.66732479167</v>
+      </c>
+      <c r="C16" s="13" t="inlineStr">
+        <is>
+          <t>חילוץ נכשל</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>חריגה ממכסת ה-API של ספק ה-AI. פרטים: gemini/gemini-3.8-flash: 429 You exceeded your current quota, please check your plan and billing details. For more information on this error, head to: https://ai.goo | gemini/gemini-3.7-flash: 429 You exceeded your current quota, please check your plan and billing details. For more information on this error, head to: https://ai.goo | gemini/gemini-3.5-flash: 429 You exceeded your current quota, please check your plan and billing details. For more information on this error, head to: https://ai.goo | gemini/gemini-3.5-flash-lite: Timeout of 60.0s exceeded, last exception: 503 This model is currently experiencing high demand. Spikes in demand are usually temporary. Ple</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>מייל נכנס</t>
+        </is>
+      </c>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t>גיא כהן &lt;mail4games21@gmail.com&gt;</t>
+        </is>
+      </c>
+      <c r="G16" s="2" t="inlineStr">
+        <is>
+          <t>בדיקת חשבונית (טסט לאוטומציה)</t>
+        </is>
+      </c>
+      <c r="H16" s="2" t="inlineStr">
+        <is>
+          <t>טופס התחשבנות 3 (תקול - אי התאמה בחישוב) - קלין-טק כביסה.pdf</t>
+        </is>
+      </c>
+      <c r="I16" s="2" t="n"/>
+      <c r="J16" s="2" t="n"/>
+      <c r="K16" s="2" t="n"/>
+      <c r="L16" s="2" t="n"/>
+      <c r="M16" s="12" t="n"/>
+      <c r="N16" s="12" t="n"/>
+      <c r="O16" s="12" t="n"/>
+      <c r="P16" s="2" t="n"/>
+      <c r="Q16" s="5" t="n"/>
+      <c r="R16" s="2" t="n"/>
+      <c r="S16" s="5" t="n"/>
+      <c r="T16" s="5" t="n"/>
+      <c r="U16" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="V16" s="2" t="n"/>
+      <c r="W16" s="2" t="inlineStr">
+        <is>
+          <t>הספק הוא תמיד א ב טכנלוגיות וניסויים (פרומפט תקול)</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="n">
+        <v>37</v>
+      </c>
+      <c r="B17" s="11" t="n">
+        <v>46293.66806519676</v>
+      </c>
+      <c r="C17" s="13" t="inlineStr">
+        <is>
+          <t>חילוץ נכשל</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>חריגה ממכסת ה-API של ספק ה-AI. פרטים: gemini/gemini-3.8-flash: 429 You exceeded your current quota, please check your plan and billing details. For more information on this error, head to: https://ai.goo | gemini/gemini-3.7-flash: 429 You exceeded your current quota, please check your plan and billing details. For more information on this error, head to: https://ai.goo | gemini/gemini-3.5-flash: 429 You exceeded your current quota, please check your plan and billing details. For more information on this error, head to: https://ai.goo | gemini/gemini-3.5-flash-lite: Timeout of 60.0s exceeded, last exception: 503 This model is currently experiencing high demand. Spikes in demand are usually temporary. Ple</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>מייל נכנס</t>
+        </is>
+      </c>
+      <c r="F17" s="2" t="inlineStr">
+        <is>
+          <t>גיא כהן &lt;mail4games21@gmail.com&gt;</t>
+        </is>
+      </c>
+      <c r="G17" s="2" t="inlineStr">
+        <is>
+          <t>בדיקת חשבונית (טסט לאוטומציה)</t>
+        </is>
+      </c>
+      <c r="H17" s="2" t="inlineStr">
+        <is>
+          <t>טופס התחשבנות 5 (תקול - טעות כפל בשורה ומע_מ שגוי) - שפע קייטרינג.pdf</t>
+        </is>
+      </c>
+      <c r="I17" s="2" t="n"/>
+      <c r="J17" s="2" t="n"/>
+      <c r="K17" s="2" t="n"/>
+      <c r="L17" s="2" t="n"/>
+      <c r="M17" s="12" t="n"/>
+      <c r="N17" s="12" t="n"/>
+      <c r="O17" s="12" t="n"/>
+      <c r="P17" s="2" t="n"/>
+      <c r="Q17" s="5" t="n"/>
+      <c r="R17" s="2" t="n"/>
+      <c r="S17" s="5" t="n"/>
+      <c r="T17" s="5" t="n"/>
+      <c r="U17" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="V17" s="2" t="n"/>
+      <c r="W17" s="2" t="inlineStr">
+        <is>
+          <t>הספק הוא תמיד א ב טכנלוגיות וניסויים (פרומפט תקול)</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="n">
+        <v>38</v>
+      </c>
+      <c r="B18" s="11" t="n">
+        <v>46293.66876641204</v>
+      </c>
+      <c r="C18" s="13" t="inlineStr">
+        <is>
+          <t>חילוץ נכשל</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>חריגה ממכסת ה-API של ספק ה-AI. פרטים: gemini/gemini-3.8-flash: 429 You exceeded your current quota, please check your plan and billing details. For more information on this error, head to: https://ai.goo | gemini/gemini-3.7-flash: 429 You exceeded your current quota, please check your plan and billing details. For more information on this error, head to: https://ai.goo | gemini/gemini-3.5-flash: 429 You exceeded your current quota, please check your plan and billing details. For more information on this error, head to: https://ai.goo | gemini/gemini-3.5-flash-lite: Timeout of 60.0s exceeded, last exception: 503 This model is currently experiencing high demand. Spikes in demand are usually temporary. Ple</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>מייל נכנס</t>
+        </is>
+      </c>
+      <c r="F18" s="2" t="inlineStr">
+        <is>
+          <t>גיא כהן &lt;mail4games21@gmail.com&gt;</t>
+        </is>
+      </c>
+      <c r="G18" s="2" t="inlineStr">
+        <is>
+          <t>בדיקת חשבונית (טסט לאוטומציה)</t>
+        </is>
+      </c>
+      <c r="H18" s="2" t="inlineStr">
+        <is>
+          <t>טופס התחשבנות ספק - מדי-פארם בע_מ.pdf</t>
+        </is>
+      </c>
+      <c r="I18" s="2" t="n"/>
+      <c r="J18" s="2" t="n"/>
+      <c r="K18" s="2" t="n"/>
+      <c r="L18" s="2" t="n"/>
+      <c r="M18" s="12" t="n"/>
+      <c r="N18" s="12" t="n"/>
+      <c r="O18" s="12" t="n"/>
+      <c r="P18" s="2" t="n"/>
+      <c r="Q18" s="5" t="n"/>
+      <c r="R18" s="2" t="n"/>
+      <c r="S18" s="5" t="n"/>
+      <c r="T18" s="5" t="n"/>
+      <c r="U18" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="V18" s="2" t="n"/>
+      <c r="W18" s="2" t="inlineStr">
+        <is>
+          <t>הספק הוא תמיד א ב טכנלוגיות וניסויים (פרומפט תקול)</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="n">
+        <v>39</v>
+      </c>
+      <c r="B19" s="11" t="n">
+        <v>46293.67565167824</v>
+      </c>
+      <c r="C19" s="13" t="inlineStr">
+        <is>
+          <t>חילוץ נכשל</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>חריגה ממכסת ה-API של ספק ה-AI. פרטים: gemini/gemini-3.8-flash: 429 You exceeded your current quota, please check your plan and billing details. For more information on this error, head to: https://ai.goo | gemini/gemini-3.7-flash: 429 You exceeded your current quota, please check your plan and billing details. For more information on this error, head to: https://ai.goo | gemini/gemini-3.5-flash: 429 You exceeded your current quota, please check your plan and billing details. For more information on this error, head to: https://ai.goo | gemini/gemini-3.5-flash-lite: Timeout of 60.0s exceeded, last exception: 503 This model is currently experiencing high demand. Spikes in demand are usually temporary. Ple</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t>מייל נכנס</t>
+        </is>
+      </c>
+      <c r="F19" s="2" t="inlineStr">
+        <is>
+          <t>גיא כהן &lt;mail4games21@gmail.com&gt;</t>
+        </is>
+      </c>
+      <c r="G19" s="2" t="inlineStr">
+        <is>
+          <t>בדיקת חשבונית (טסט לאוטומציה)</t>
+        </is>
+      </c>
+      <c r="H19" s="2" t="inlineStr">
+        <is>
+          <t>טופס התחשבנות 4 (תקול - חוסר שדות וערכים לא מספריים) - א.ב. מיזוג.pdf</t>
+        </is>
+      </c>
+      <c r="I19" s="2" t="n"/>
+      <c r="J19" s="2" t="n"/>
+      <c r="K19" s="2" t="n"/>
+      <c r="L19" s="2" t="n"/>
+      <c r="M19" s="12" t="n"/>
+      <c r="N19" s="12" t="n"/>
+      <c r="O19" s="12" t="n"/>
+      <c r="P19" s="2" t="n"/>
+      <c r="Q19" s="5" t="n"/>
+      <c r="R19" s="2" t="n"/>
+      <c r="S19" s="5" t="n"/>
+      <c r="T19" s="5" t="n"/>
+      <c r="U19" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="V19" s="2" t="n"/>
+      <c r="W19" s="2" t="inlineStr">
+        <is>
+          <t>הספק הוא תמיד א ב טכנלוגיות וניסויים (פרומפט תקול)</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="n">
+        <v>40</v>
+      </c>
+      <c r="B20" s="11" t="n">
+        <v>46293.67658344907</v>
+      </c>
+      <c r="C20" s="13" t="inlineStr">
+        <is>
+          <t>חילוץ נכשל</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>חריגה ממכסת ה-API של ספק ה-AI. פרטים: gemini/gemini-3.8-flash: 429 You exceeded your current quota, please check your plan and billing details. For more information on this error, head to: https://ai.goo | gemini/gemini-3.7-flash: 429 You exceeded your current quota, please check your plan and billing details. For more information on this error, head to: https://ai.goo | gemini/gemini-3.5-flash: 429 You exceeded your current quota, please check your plan and billing details. For more information on this error, head to: https://ai.goo | gemini/gemini-3.5-flash-lite: Timeout of 60.0s exceeded, last exception: 503 This model is currently experiencing high demand. Spikes in demand are usually temporary. Ple</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>מייל נכנס</t>
+        </is>
+      </c>
+      <c r="F20" s="2" t="inlineStr">
+        <is>
+          <t>גיא כהן &lt;mail4games21@gmail.com&gt;</t>
+        </is>
+      </c>
+      <c r="G20" s="2" t="inlineStr">
+        <is>
+          <t>בדיקת חשבונית (טסט לאוטומציה)</t>
+        </is>
+      </c>
+      <c r="H20" s="2" t="inlineStr">
+        <is>
+          <t>טופס התחשבנות 2 (תקין - עיצוב שונה) - ש.ל.ה הסעות רפואיות.pdf</t>
+        </is>
+      </c>
+      <c r="I20" s="2" t="n"/>
+      <c r="J20" s="2" t="n"/>
+      <c r="K20" s="2" t="n"/>
+      <c r="L20" s="2" t="n"/>
+      <c r="M20" s="12" t="n"/>
+      <c r="N20" s="12" t="n"/>
+      <c r="O20" s="12" t="n"/>
+      <c r="P20" s="2" t="n"/>
+      <c r="Q20" s="5" t="n"/>
+      <c r="R20" s="2" t="n"/>
+      <c r="S20" s="5" t="n"/>
+      <c r="T20" s="5" t="n"/>
+      <c r="U20" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="V20" s="2" t="n"/>
+      <c r="W20" s="2" t="inlineStr">
+        <is>
+          <t>הספק הוא תמיד א ב טכנלוגיות וניסויים (פרומפט תקול)</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="n">
+        <v>41</v>
+      </c>
+      <c r="B21" s="11" t="n">
+        <v>46293.6768666088</v>
+      </c>
+      <c r="C21" s="13" t="inlineStr">
+        <is>
+          <t>חילוץ נכשל</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>חריגה ממכסת ה-API של ספק ה-AI. פרטים: gemini/gemini-3.8-flash: 429 You exceeded your current quota, please check your plan and billing details. For more information on this error, head to: https://ai.goo | gemini/gemini-3.7-flash: 429 You exceeded your current quota, please check your plan and billing details. For more information on this error, head to: https://ai.goo | gemini/gemini-3.5-flash: 429 You exceeded your current quota, please check your plan and billing details. For more information on this error, head to: https://ai.goo | gemini/gemini-3.5-flash-lite: 429 You exceeded your current quota, please check your plan and billing details. For more information on this error, head to: https://ai.goo</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="inlineStr">
+        <is>
+          <t>מייל נכנס</t>
+        </is>
+      </c>
+      <c r="F21" s="2" t="inlineStr">
+        <is>
+          <t>גיא כהן &lt;mail4games21@gmail.com&gt;</t>
+        </is>
+      </c>
+      <c r="G21" s="2" t="inlineStr">
+        <is>
+          <t>בדיקת חשבונית (טסט לאוטומציה)</t>
+        </is>
+      </c>
+      <c r="H21" s="2" t="inlineStr">
+        <is>
+          <t>טופס התחשבנות 4 (תקול - חוסר שדות וערכים לא מספריים) - א.ב. מיזוג.pdf</t>
+        </is>
+      </c>
+      <c r="I21" s="2" t="n"/>
+      <c r="J21" s="2" t="n"/>
+      <c r="K21" s="2" t="n"/>
+      <c r="L21" s="2" t="n"/>
+      <c r="M21" s="12" t="n"/>
+      <c r="N21" s="12" t="n"/>
+      <c r="O21" s="12" t="n"/>
+      <c r="P21" s="2" t="n"/>
+      <c r="Q21" s="5" t="n"/>
+      <c r="R21" s="2" t="n"/>
+      <c r="S21" s="5" t="n"/>
+      <c r="T21" s="5" t="n"/>
+      <c r="U21" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="V21" s="2" t="n"/>
+      <c r="W21" s="2" t="inlineStr">
+        <is>
+          <t>הספק הוא תמיד א ב טכנלוגיות וניסויים (פרומפט תקול)</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="n">
+        <v>42</v>
+      </c>
+      <c r="B22" s="11" t="n">
+        <v>46293.67731612269</v>
+      </c>
+      <c r="C22" s="13" t="inlineStr">
+        <is>
+          <t>חילוץ נכשל</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>חריגה ממכסת ה-API של ספק ה-AI. פרטים: gemini/gemini-3.8-flash: 429 You exceeded your current quota, please check your plan and billing details. For more information on this error, head to: https://ai.goo | gemini/gemini-3.7-flash: 429 You exceeded your current quota, please check your plan and billing details. For more information on this error, head to: https://ai.goo | gemini/gemini-3.5-flash: 429 You exceeded your current quota, please check your plan and billing details. For more information on this error, head to: https://ai.goo | gemini/gemini-3.5-flash-lite: 429 You exceeded your current quota, please check your plan and billing details. For more information on this error, head to: https://ai.goo</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t>מייל נכנס</t>
+        </is>
+      </c>
+      <c r="F22" s="2" t="inlineStr">
+        <is>
+          <t>גיא כהן &lt;mail4games21@gmail.com&gt;</t>
+        </is>
+      </c>
+      <c r="G22" s="2" t="inlineStr">
+        <is>
+          <t>בדיקת חשבונית (טסט לאוטומציה)</t>
+        </is>
+      </c>
+      <c r="H22" s="2" t="inlineStr">
+        <is>
+          <t>טופס התחשבנות 3 (תקול - אי התאמה בחישוב) - קלין-טק כביסה.pdf</t>
+        </is>
+      </c>
+      <c r="I22" s="2" t="n"/>
+      <c r="J22" s="2" t="n"/>
+      <c r="K22" s="2" t="n"/>
+      <c r="L22" s="2" t="n"/>
+      <c r="M22" s="12" t="n"/>
+      <c r="N22" s="12" t="n"/>
+      <c r="O22" s="12" t="n"/>
+      <c r="P22" s="2" t="n"/>
+      <c r="Q22" s="5" t="n"/>
+      <c r="R22" s="2" t="n"/>
+      <c r="S22" s="5" t="n"/>
+      <c r="T22" s="5" t="n"/>
+      <c r="U22" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="V22" s="2" t="n"/>
+      <c r="W22" s="2" t="inlineStr">
+        <is>
+          <t>הספק הוא תמיד א ב טכנלוגיות וניסויים (פרומפט תקול)</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="n">
+        <v>43</v>
+      </c>
+      <c r="B23" s="11" t="n">
+        <v>46293.67737708333</v>
+      </c>
+      <c r="C23" s="13" t="inlineStr">
+        <is>
+          <t>חילוץ נכשל</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t>החילוץ נכשל בכל ספקי ה-AI. פרטים: gemini/-: [SSL] record layer failure (_ssl.c:2590)</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="inlineStr">
+        <is>
+          <t>מייל נכנס</t>
+        </is>
+      </c>
+      <c r="F23" s="2" t="inlineStr">
+        <is>
+          <t>גיא כהן &lt;mail4games21@gmail.com&gt;</t>
+        </is>
+      </c>
+      <c r="G23" s="2" t="inlineStr">
+        <is>
+          <t>בדיקת חשבונית (טסט לאוטומציה)</t>
+        </is>
+      </c>
+      <c r="H23" s="2" t="inlineStr">
+        <is>
+          <t>טופס התחשבנות 5 (תקול - טעות כפל בשורה ומע_מ שגוי) - שפע קייטרינג.pdf</t>
+        </is>
+      </c>
+      <c r="I23" s="2" t="n"/>
+      <c r="J23" s="2" t="n"/>
+      <c r="K23" s="2" t="n"/>
+      <c r="L23" s="2" t="n"/>
+      <c r="M23" s="12" t="n"/>
+      <c r="N23" s="12" t="n"/>
+      <c r="O23" s="12" t="n"/>
+      <c r="P23" s="2" t="n"/>
+      <c r="Q23" s="5" t="n"/>
+      <c r="R23" s="2" t="n"/>
+      <c r="S23" s="5" t="n"/>
+      <c r="T23" s="5" t="n"/>
+      <c r="U23" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="V23" s="2" t="n"/>
+      <c r="W23" s="2" t="inlineStr">
+        <is>
+          <t>הספק הוא תמיד א ב טכנלוגיות וניסויים (פרומפט תקול)</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="n">
+        <v>44</v>
+      </c>
+      <c r="B24" s="11" t="n">
+        <v>46293.67732210648</v>
+      </c>
+      <c r="C24" s="13" t="inlineStr">
+        <is>
+          <t>חילוץ נכשל</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>החילוץ נכשל בכל ספקי ה-AI. פרטים: gemini/-: [SSL] record layer failure (_ssl.c:2590)</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="inlineStr">
+        <is>
+          <t>מייל נכנס</t>
+        </is>
+      </c>
+      <c r="F24" s="2" t="inlineStr">
+        <is>
+          <t>גיא כהן &lt;mail4games21@gmail.com&gt;</t>
+        </is>
+      </c>
+      <c r="G24" s="2" t="inlineStr">
+        <is>
+          <t>בדיקת חשבונית (טסט לאוטומציה)</t>
+        </is>
+      </c>
+      <c r="H24" s="2" t="inlineStr">
+        <is>
+          <t>טופס התחשבנות 2 (תקין - עיצוב שונה) - ש.ל.ה הסעות רפואיות.pdf</t>
+        </is>
+      </c>
+      <c r="I24" s="2" t="n"/>
+      <c r="J24" s="2" t="n"/>
+      <c r="K24" s="2" t="n"/>
+      <c r="L24" s="2" t="n"/>
+      <c r="M24" s="12" t="n"/>
+      <c r="N24" s="12" t="n"/>
+      <c r="O24" s="12" t="n"/>
+      <c r="P24" s="2" t="n"/>
+      <c r="Q24" s="5" t="n"/>
+      <c r="R24" s="2" t="n"/>
+      <c r="S24" s="5" t="n"/>
+      <c r="T24" s="5" t="n"/>
+      <c r="U24" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="V24" s="2" t="n"/>
+      <c r="W24" s="2" t="inlineStr">
+        <is>
+          <t>הספק הוא תמיד א ב טכנלוגיות וניסויים (פרומפט תקול)</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="n">
+        <v>45</v>
+      </c>
+      <c r="B25" s="11" t="n">
+        <v>46293.67745412037</v>
+      </c>
+      <c r="C25" s="13" t="inlineStr">
+        <is>
+          <t>חילוץ נכשל</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="inlineStr">
+        <is>
+          <t>חריגה ממכסת ה-API של ספק ה-AI. פרטים: gemini/gemini-3.8-flash: 429 You exceeded your current quota, please check your plan and billing details. For more information on this error, head to: https://ai.goo | gemini/gemini-3.7-flash: 429 You exceeded your current quota, please check your plan and billing details. For more information on this error, head to: https://ai.goo | gemini/gemini-3.5-flash: 429 You exceeded your current quota, please check your plan and billing details. For more information on this error, head to: https://ai.goo | gemini/gemini-3.5-flash-lite: 429 You exceeded your current quota, please check your plan and billing details. For more information on this error, head to: https://ai.goo</t>
+        </is>
+      </c>
+      <c r="E25" s="2" t="inlineStr">
+        <is>
+          <t>מייל נכנס</t>
+        </is>
+      </c>
+      <c r="F25" s="2" t="inlineStr">
+        <is>
+          <t>גיא כהן &lt;mail4games21@gmail.com&gt;</t>
+        </is>
+      </c>
+      <c r="G25" s="2" t="inlineStr">
+        <is>
+          <t>בדיקת חשבונית (טסט לאוטומציה)</t>
+        </is>
+      </c>
+      <c r="H25" s="2" t="inlineStr">
+        <is>
+          <t>טופס התחשבנות ספק - מדי-פארם בע_מ.pdf</t>
+        </is>
+      </c>
+      <c r="I25" s="2" t="n"/>
+      <c r="J25" s="2" t="n"/>
+      <c r="K25" s="2" t="n"/>
+      <c r="L25" s="2" t="n"/>
+      <c r="M25" s="12" t="n"/>
+      <c r="N25" s="12" t="n"/>
+      <c r="O25" s="12" t="n"/>
+      <c r="P25" s="2" t="n"/>
+      <c r="Q25" s="5" t="n"/>
+      <c r="R25" s="2" t="n"/>
+      <c r="S25" s="5" t="n"/>
+      <c r="T25" s="5" t="n"/>
+      <c r="U25" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="V25" s="2" t="n"/>
+      <c r="W25" s="2" t="inlineStr">
+        <is>
+          <t>הספק הוא תמיד א ב טכנלוגיות וניסויים (פרומפט תקול)</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="n">
+        <v>46</v>
+      </c>
+      <c r="B26" s="11" t="n">
+        <v>46293.67745496528</v>
+      </c>
+      <c r="C26" s="13" t="inlineStr">
+        <is>
+          <t>חילוץ נכשל</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>חריגה ממכסת ה-API של ספק ה-AI. פרטים: gemini/gemini-3.8-flash: 429 You exceeded your current quota, please check your plan and billing details. For more information on this error, head to: https://ai.goo | gemini/gemini-3.7-flash: 429 You exceeded your current quota, please check your plan and billing details. For more information on this error, head to: https://ai.goo | gemini/gemini-3.5-flash: 429 You exceeded your current quota, please check your plan and billing details. For more information on this error, head to: https://ai.goo | gemini/gemini-3.5-flash-lite: 504 Deadline expired before operation could complete.</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="inlineStr">
+        <is>
+          <t>מייל נכנס</t>
+        </is>
+      </c>
+      <c r="F26" s="2" t="inlineStr">
+        <is>
+          <t>גיא כהן &lt;mail4games21@gmail.com&gt;</t>
+        </is>
+      </c>
+      <c r="G26" s="2" t="inlineStr">
+        <is>
+          <t>בדיקת חשבונית (טסט לאוטומציה)</t>
+        </is>
+      </c>
+      <c r="H26" s="2" t="inlineStr">
+        <is>
+          <t>טופס התחשבנות 3 (תקול - אי התאמה בחישוב) - קלין-טק כביסה.pdf</t>
+        </is>
+      </c>
+      <c r="I26" s="2" t="n"/>
+      <c r="J26" s="2" t="n"/>
+      <c r="K26" s="2" t="n"/>
+      <c r="L26" s="2" t="n"/>
+      <c r="M26" s="12" t="n"/>
+      <c r="N26" s="12" t="n"/>
+      <c r="O26" s="12" t="n"/>
+      <c r="P26" s="2" t="n"/>
+      <c r="Q26" s="5" t="n"/>
+      <c r="R26" s="2" t="n"/>
+      <c r="S26" s="5" t="n"/>
+      <c r="T26" s="5" t="n"/>
+      <c r="U26" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="V26" s="2" t="n"/>
+      <c r="W26" s="2" t="inlineStr">
+        <is>
+          <t>הספק הוא תמיד א ב טכנלוגיות וניסויים (פרומפט תקול)</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="n">
+        <v>47</v>
+      </c>
+      <c r="B27" s="11" t="n">
+        <v>46293.6789083912</v>
+      </c>
+      <c r="C27" s="13" t="inlineStr">
+        <is>
+          <t>חילוץ נכשל</t>
+        </is>
+      </c>
+      <c r="D27" s="2" t="inlineStr">
+        <is>
+          <t>חריגה ממכסת ה-API של ספק ה-AI. פרטים: gemini/gemini-3.8-flash: 429 You exceeded your current quota, please check your plan and billing details. For more information on this error, head to: https://ai.goo | gemini/gemini-3.7-flash: 429 You exceeded your current quota, please check your plan and billing details. For more information on this error, head to: https://ai.goo | gemini/gemini-3.5-flash: 429 You exceeded your current quota, please check your plan and billing details. For more information on this error, head to: https://ai.goo | gemini/gemini-3.5-flash-lite: 504 Deadline Exceeded</t>
+        </is>
+      </c>
+      <c r="E27" s="2" t="inlineStr">
+        <is>
+          <t>מייל נכנס</t>
+        </is>
+      </c>
+      <c r="F27" s="2" t="inlineStr">
+        <is>
+          <t>גיא כהן &lt;mail4games21@gmail.com&gt;</t>
+        </is>
+      </c>
+      <c r="G27" s="2" t="inlineStr">
+        <is>
+          <t>בדיקת חשבונית (טסט לאוטומציה)</t>
+        </is>
+      </c>
+      <c r="H27" s="2" t="inlineStr">
+        <is>
+          <t>טופס התחשבנות 5 (תקול - טעות כפל בשורה ומע_מ שגוי) - שפע קייטרינג.pdf</t>
+        </is>
+      </c>
+      <c r="I27" s="2" t="n"/>
+      <c r="J27" s="2" t="n"/>
+      <c r="K27" s="2" t="n"/>
+      <c r="L27" s="2" t="n"/>
+      <c r="M27" s="12" t="n"/>
+      <c r="N27" s="12" t="n"/>
+      <c r="O27" s="12" t="n"/>
+      <c r="P27" s="2" t="n"/>
+      <c r="Q27" s="5" t="n"/>
+      <c r="R27" s="2" t="n"/>
+      <c r="S27" s="5" t="n"/>
+      <c r="T27" s="5" t="n"/>
+      <c r="U27" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="V27" s="2" t="n"/>
+      <c r="W27" s="2" t="inlineStr">
+        <is>
+          <t>הספק הוא תמיד א ב טכנלוגיות וניסויים (פרומפט תקול)</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="n">
+        <v>48</v>
+      </c>
+      <c r="B28" s="11" t="n">
+        <v>46293.67964604167</v>
+      </c>
+      <c r="C28" s="13" t="inlineStr">
+        <is>
+          <t>חילוץ נכשל</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="inlineStr">
+        <is>
+          <t>חריגה ממכסת ה-API של ספק ה-AI. פרטים: gemini/gemini-3.8-flash: 429 You exceeded your current quota, please check your plan and billing details. For more information on this error, head to: https://ai.goo | gemini/gemini-3.7-flash: 429 You exceeded your current quota, please check your plan and billing details. For more information on this error, head to: https://ai.goo | gemini/gemini-3.5-flash: 429 You exceeded your current quota, please check your plan and billing details. For more information on this error, head to: https://ai.goo | gemini/gemini-3.5-flash-lite: Timeout of 60.0s exceeded, last exception: 503 This model is currently experiencing high demand. Spikes in demand are usually temporary. Ple</t>
+        </is>
+      </c>
+      <c r="E28" s="2" t="inlineStr">
+        <is>
+          <t>מייל נכנס</t>
+        </is>
+      </c>
+      <c r="F28" s="2" t="inlineStr">
+        <is>
+          <t>גיא כהן &lt;mail4games21@gmail.com&gt;</t>
+        </is>
+      </c>
+      <c r="G28" s="2" t="inlineStr">
+        <is>
+          <t>בדיקת חשבונית (טסט לאוטומציה)</t>
+        </is>
+      </c>
+      <c r="H28" s="2" t="inlineStr">
+        <is>
+          <t>טופס התחשבנות ספק - מדי-פארם בע_מ.pdf</t>
+        </is>
+      </c>
+      <c r="I28" s="2" t="n"/>
+      <c r="J28" s="2" t="n"/>
+      <c r="K28" s="2" t="n"/>
+      <c r="L28" s="2" t="n"/>
+      <c r="M28" s="12" t="n"/>
+      <c r="N28" s="12" t="n"/>
+      <c r="O28" s="12" t="n"/>
+      <c r="P28" s="2" t="n"/>
+      <c r="Q28" s="5" t="n"/>
+      <c r="R28" s="2" t="n"/>
+      <c r="S28" s="5" t="n"/>
+      <c r="T28" s="5" t="n"/>
+      <c r="U28" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="V28" s="2" t="n"/>
+      <c r="W28" s="2" t="inlineStr">
+        <is>
+          <t>הספק הוא תמיד א ב טכנלוגיות וניסויים (פרומפט תקול)</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="n">
+        <v>49</v>
+      </c>
+      <c r="B29" s="11" t="n">
+        <v>46293.68318603012</v>
+      </c>
+      <c r="C29" s="13" t="inlineStr">
+        <is>
+          <t>חילוץ נכשל</t>
+        </is>
+      </c>
+      <c r="D29" s="2" t="inlineStr">
+        <is>
+          <t>חריגה ממכסת ה-API של ספק ה-AI. פרטים: gemini/gemini-3.8-flash: 429 You exceeded your current quota, please check your plan and billing details. For more information on this error, head to: https://ai.goo | gemini/gemini-3.7-flash: 429 You exceeded your current quota, please check your plan and billing details. For more information on this error, head to: https://ai.goo | gemini/gemini-3.5-flash: 429 You exceeded your current quota, please check your plan and billing details. For more information on this error, head to: https://ai.goo | gemini/gemini-3.5-flash-lite: 504 Deadline expired before operation could complete.</t>
+        </is>
+      </c>
+      <c r="E29" s="2" t="inlineStr">
+        <is>
+          <t>העלאה ידנית</t>
+        </is>
+      </c>
+      <c r="F29" s="2" t="n"/>
+      <c r="G29" s="2" t="n"/>
+      <c r="H29" s="2" t="inlineStr">
+        <is>
+          <t>טופס התחשבנות 5 (תקול - טעות כפל בשורה ומע_מ שגוי) - שפע קייטרינג.pdf</t>
+        </is>
+      </c>
+      <c r="I29" s="2" t="n"/>
+      <c r="J29" s="2" t="n"/>
+      <c r="K29" s="2" t="n"/>
+      <c r="L29" s="2" t="n"/>
+      <c r="M29" s="12" t="n"/>
+      <c r="N29" s="12" t="n"/>
+      <c r="O29" s="12" t="n"/>
+      <c r="P29" s="2" t="n"/>
+      <c r="Q29" s="5" t="n"/>
+      <c r="R29" s="2" t="n"/>
+      <c r="S29" s="5" t="n"/>
+      <c r="T29" s="5" t="n"/>
+      <c r="U29" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="V29" s="2" t="n"/>
+      <c r="W29" s="2" t="inlineStr">
+        <is>
+          <t>הספק הוא תמיד א ב טכנלוגיות וניסויים (פרומפט תקול)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:W9"/>
+  <autoFilter ref="A1:W29"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
feat: add Google Gemini extraction provider with model fallback and centralized configuration
</commit_message>
<xml_diff>
--- a/data/GoldenCare_Master.xlsx
+++ b/data/GoldenCare_Master.xlsx
@@ -10,8 +10,8 @@
     <sheet name="שורות חיוב" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'מסמכים'!$A$1:$W$29</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'שורות חיוב'!$A$1:$J$95</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'מסמכים'!$A$1:$W$32</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'שורות חיוב'!$A$1:$J$98</definedName>
   </definedNames>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
@@ -19,10 +19,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="3">
+  <numFmts count="4">
     <numFmt numFmtId="164" formatCode="DD/MM/YYYY HH:MM"/>
     <numFmt numFmtId="165" formatCode="DD/MM/YYYY"/>
     <numFmt numFmtId="166" formatCode="yyyy-mm-dd h:mm:ss"/>
+    <numFmt numFmtId="167" formatCode="yyyy-mm-dd"/>
   </numFmts>
   <fonts count="2">
     <font>
@@ -490,7 +491,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:W29"/>
+  <dimension ref="A1:W32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -2482,7 +2483,7 @@
         <v>49</v>
       </c>
       <c r="B29" s="11" t="n">
-        <v>46293.68318603012</v>
+        <v>46293.6831860301</v>
       </c>
       <c r="C29" s="13" t="inlineStr">
         <is>
@@ -2528,8 +2529,195 @@
         </is>
       </c>
     </row>
+    <row r="30">
+      <c r="A30" s="2" t="n">
+        <v>50</v>
+      </c>
+      <c r="B30" s="11" t="n">
+        <v>46293.6914303588</v>
+      </c>
+      <c r="C30" s="13" t="inlineStr">
+        <is>
+          <t>חילוץ נכשל</t>
+        </is>
+      </c>
+      <c r="D30" s="2" t="inlineStr">
+        <is>
+          <t>חריגה ממכסת ה-API של ספק ה-AI. פרטים: gemini/gemini-3.8-flash: 429 You exceeded your current quota, please check your plan and billing details. For more information on this error, head to: https://ai.goo | gemini/gemini-3.7-flash: 429 You exceeded your current quota, please check your plan and billing details. For more information on this error, head to: https://ai.goo | gemini/gemini-3.5-flash: 429 You exceeded your current quota, please check your plan and billing details. For more information on this error, head to: https://ai.goo | gemini/gemini-3.5-flash-lite: Timeout of 60.0s exceeded, last exception: 503 This model is currently experiencing high demand. Spikes in demand are usually temporary. Ple | gemini/gemini-1.5-pro: 404 models/gemini-1.5-pro is not found for API version v1beta, or is not supported for generateContent. Call ModelService.ListModels to see  | gemini/gemini-1.5-flash: 404 models/gemini-1.5-flash is not found for API version v1beta, or is not supported for generateContent. Call ModelService.ListModels to se | gemini/gemini-1.5-flash-8b: 404 models/gemini-1.5-flash-8b is not found for API version v1beta, or is not supported for generateContent. Call ModelService.ListModels to</t>
+        </is>
+      </c>
+      <c r="E30" s="2" t="inlineStr">
+        <is>
+          <t>העלאה ידנית</t>
+        </is>
+      </c>
+      <c r="F30" s="2" t="n"/>
+      <c r="G30" s="2" t="n"/>
+      <c r="H30" s="2" t="inlineStr">
+        <is>
+          <t>טופס התחשבנות 2 (תקין - עיצוב שונה) - ש.ל.ה הסעות רפואיות.pdf</t>
+        </is>
+      </c>
+      <c r="I30" s="2" t="n"/>
+      <c r="J30" s="2" t="n"/>
+      <c r="K30" s="2" t="n"/>
+      <c r="L30" s="2" t="n"/>
+      <c r="M30" s="12" t="n"/>
+      <c r="N30" s="12" t="n"/>
+      <c r="O30" s="12" t="n"/>
+      <c r="P30" s="2" t="n"/>
+      <c r="Q30" s="5" t="n"/>
+      <c r="R30" s="2" t="n"/>
+      <c r="S30" s="5" t="n"/>
+      <c r="T30" s="5" t="n"/>
+      <c r="U30" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="V30" s="2" t="n"/>
+      <c r="W30" s="2" t="inlineStr">
+        <is>
+          <t>הספק הוא תמיד א ב טכנלוגיות וניסויים (פרומפט תקול)</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="n">
+        <v>51</v>
+      </c>
+      <c r="B31" s="11" t="n">
+        <v>46293.69504575231</v>
+      </c>
+      <c r="C31" s="13" t="inlineStr">
+        <is>
+          <t>חילוץ נכשל</t>
+        </is>
+      </c>
+      <c r="D31" s="2" t="inlineStr">
+        <is>
+          <t>חריגה ממכסת ה-API של ספק ה-AI. פרטים: gemini/gemini-3.8-flash: 429 You exceeded your current quota, please check your plan and billing details. For more information on this error, head to: https://ai.goo | gemini/gemini-3.7-flash: 429 You exceeded your current quota, please check your plan and billing details. For more information on this error, head to: https://ai.goo | gemini/gemini-3.5-flash: 429 You exceeded your current quota, please check your plan and billing details. For more information on this error, head to: https://ai.goo | gemini/gemini-3.5-flash-lite: Timeout of 60.0s exceeded, last exception: 503 This model is currently experiencing high demand. Spikes in demand are usually temporary. Ple | gemini/gemini-1.5-pro: 404 models/gemini-1.5-pro is not found for API version v1beta, or is not supported for generateContent. Call ModelService.ListModels to see  | gemini/gemini-1.5-flash: 404 models/gemini-1.5-flash is not found for API version v1beta, or is not supported for generateContent. Call ModelService.ListModels to se | gemini/gemini-1.5-flash-8b: 404 models/gemini-1.5-flash-8b is not found for API version v1beta, or is not supported for generateContent. Call ModelService.ListModels to</t>
+        </is>
+      </c>
+      <c r="E31" s="2" t="inlineStr">
+        <is>
+          <t>העלאה ידנית</t>
+        </is>
+      </c>
+      <c r="F31" s="2" t="n"/>
+      <c r="G31" s="2" t="n"/>
+      <c r="H31" s="2" t="inlineStr">
+        <is>
+          <t>טופס התחשבנות 2 (תקין - עיצוב שונה) - ש.ל.ה הסעות רפואיות.pdf</t>
+        </is>
+      </c>
+      <c r="I31" s="2" t="n"/>
+      <c r="J31" s="2" t="n"/>
+      <c r="K31" s="2" t="n"/>
+      <c r="L31" s="2" t="n"/>
+      <c r="M31" s="12" t="n"/>
+      <c r="N31" s="12" t="n"/>
+      <c r="O31" s="12" t="n"/>
+      <c r="P31" s="2" t="n"/>
+      <c r="Q31" s="5" t="n"/>
+      <c r="R31" s="2" t="n"/>
+      <c r="S31" s="5" t="n"/>
+      <c r="T31" s="5" t="n"/>
+      <c r="U31" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="V31" s="2" t="n"/>
+      <c r="W31" s="2" t="inlineStr">
+        <is>
+          <t>הספק הוא תמיד א ב טכנלוגיות וניסויים (פרומפט תקול)</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="n">
+        <v>52</v>
+      </c>
+      <c r="B32" s="11" t="n">
+        <v>46293.69722997623</v>
+      </c>
+      <c r="C32" s="9" t="inlineStr">
+        <is>
+          <t>תקין</t>
+        </is>
+      </c>
+      <c r="D32" s="2" t="inlineStr"/>
+      <c r="E32" s="2" t="inlineStr">
+        <is>
+          <t>העלאה ידנית</t>
+        </is>
+      </c>
+      <c r="F32" s="2" t="n"/>
+      <c r="G32" s="2" t="n"/>
+      <c r="H32" s="2" t="inlineStr">
+        <is>
+          <t>טופס התחשבנות 2 (תקין - עיצוב שונה) - ש.ל.ה הסעות רפואיות.pdf</t>
+        </is>
+      </c>
+      <c r="I32" s="2" t="inlineStr">
+        <is>
+          <t>ש.ל.ה שירותי לוגיסטיקה והסעות רפואיות בע"מ</t>
+        </is>
+      </c>
+      <c r="J32" s="2" t="inlineStr">
+        <is>
+          <t>512998410</t>
+        </is>
+      </c>
+      <c r="K32" s="2" t="inlineStr">
+        <is>
+          <t>ריכוז חיובים חודשי / דרישת תשלום</t>
+        </is>
+      </c>
+      <c r="L32" s="2" t="inlineStr">
+        <is>
+          <t>SLH-88421</t>
+        </is>
+      </c>
+      <c r="M32" s="12" t="n">
+        <v>46264</v>
+      </c>
+      <c r="N32" s="12" t="n">
+        <v>46235</v>
+      </c>
+      <c r="O32" s="12" t="n">
+        <v>46265</v>
+      </c>
+      <c r="P32" s="2" t="inlineStr">
+        <is>
+          <t>ILS</t>
+        </is>
+      </c>
+      <c r="Q32" s="5" t="n">
+        <v>11000</v>
+      </c>
+      <c r="R32" s="2" t="n">
+        <v>17</v>
+      </c>
+      <c r="S32" s="5" t="n">
+        <v>1870</v>
+      </c>
+      <c r="T32" s="5" t="n">
+        <v>12870</v>
+      </c>
+      <c r="U32" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="V32" s="2" t="inlineStr">
+        <is>
+          <t>gemini/gemini-3.1-flash-lite</t>
+        </is>
+      </c>
+      <c r="W32" s="2" t="inlineStr">
+        <is>
+          <t>הספק הוא תמיד א ב טכנלוגיות וניסויים (פרומפט תקול)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:W29"/>
+  <autoFilter ref="A1:W32"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -2540,7 +2728,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J95"/>
+  <dimension ref="A1:J98"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -6319,8 +6507,128 @@
         </is>
       </c>
     </row>
+    <row r="96">
+      <c r="A96" s="2" t="n">
+        <v>52</v>
+      </c>
+      <c r="B96" s="2" t="inlineStr">
+        <is>
+          <t>ש.ל.ה שירותי לוגיסטיקה והסעות רפואיות בע"מ</t>
+        </is>
+      </c>
+      <c r="C96" s="2" t="inlineStr">
+        <is>
+          <t>SLH-88421</t>
+        </is>
+      </c>
+      <c r="D96" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E96" s="12" t="n">
+        <v>46239</v>
+      </c>
+      <c r="F96" s="2" t="inlineStr">
+        <is>
+          <t>הסעת מטופלים בכיסאות גלגלים (אמבולנס מותאם) קו מרכז גריאטרי גולדנקייר ← מרפאות חוץ שיבא תל השומר</t>
+        </is>
+      </c>
+      <c r="G96" s="2" t="n">
+        <v>18</v>
+      </c>
+      <c r="H96" s="5" t="n">
+        <v>350</v>
+      </c>
+      <c r="I96" s="5" t="n">
+        <v>6300</v>
+      </c>
+      <c r="J96" s="2" t="inlineStr">
+        <is>
+          <t>תקין</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="2" t="n">
+        <v>52</v>
+      </c>
+      <c r="B97" s="2" t="inlineStr">
+        <is>
+          <t>ש.ל.ה שירותי לוגיסטיקה והסעות רפואיות בע"מ</t>
+        </is>
+      </c>
+      <c r="C97" s="2" t="inlineStr">
+        <is>
+          <t>SLH-88421</t>
+        </is>
+      </c>
+      <c r="D97" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="E97" s="12" t="n">
+        <v>46248</v>
+      </c>
+      <c r="F97" s="2" t="inlineStr">
+        <is>
+          <t>שינוע דגימות מעבדה וציוד סטרילי בקירור (2–8 מעלות) איסוף יומי מרוכז מכלל מחלקות האשפוז והעברה למעבדה מרכזית</t>
+        </is>
+      </c>
+      <c r="G97" s="2" t="n">
+        <v>22</v>
+      </c>
+      <c r="H97" s="5" t="n">
+        <v>150</v>
+      </c>
+      <c r="I97" s="5" t="n">
+        <v>3300</v>
+      </c>
+      <c r="J97" s="2" t="inlineStr">
+        <is>
+          <t>תקין</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" s="2" t="n">
+        <v>52</v>
+      </c>
+      <c r="B98" s="2" t="inlineStr">
+        <is>
+          <t>ש.ל.ה שירותי לוגיסטיקה והסעות רפואיות בע"מ</t>
+        </is>
+      </c>
+      <c r="C98" s="2" t="inlineStr">
+        <is>
+          <t>SLH-88421</t>
+        </is>
+      </c>
+      <c r="D98" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="E98" s="12" t="n">
+        <v>46259</v>
+      </c>
+      <c r="F98" s="2" t="inlineStr">
+        <is>
+          <t>הזנקת חירום לילית – פינוי מטופל בליווי חובש כולל תוספת תעריף לילה והמתנת צוות רפואי בחדר מיון איכילוב</t>
+        </is>
+      </c>
+      <c r="G98" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="H98" s="5" t="n">
+        <v>700</v>
+      </c>
+      <c r="I98" s="5" t="n">
+        <v>1400</v>
+      </c>
+      <c r="J98" s="2" t="inlineStr">
+        <is>
+          <t>תקין</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J95"/>
+  <autoFilter ref="A1:J98"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
chore: add GoldenCare_Master.xlsx to data directory
</commit_message>
<xml_diff>
--- a/data/GoldenCare_Master.xlsx
+++ b/data/GoldenCare_Master.xlsx
@@ -11,8 +11,8 @@
     <sheet name="שורות חיוב" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'מסמכים'!$A$1:$W$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'שורות חיוב'!$A$1:$J$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'מסמכים'!$A$1:$W$6</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'שורות חיוב'!$A$1:$J$18</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -20,7 +20,12 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
+  <numFmts count="4">
+    <numFmt numFmtId="164" formatCode="DD/MM/YYYY HH:MM"/>
+    <numFmt numFmtId="165" formatCode="DD/MM/YYYY"/>
+    <numFmt numFmtId="166" formatCode="yyyy-mm-dd h:mm:ss"/>
+    <numFmt numFmtId="167" formatCode="yyyy-mm-dd"/>
+  </numFmts>
   <fonts count="2">
     <font>
       <name val="Calibri"/>
@@ -34,7 +39,7 @@
       <color rgb="00FFFFFF"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -44,6 +49,16 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="001F3864"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00C6EFCE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFEB9C"/>
       </patternFill>
     </fill>
   </fills>
@@ -59,10 +74,28 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="4" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -429,7 +462,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:W1"/>
+  <dimension ref="A1:W6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -574,8 +607,476 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" s="2" t="n">
+        <v>54</v>
+      </c>
+      <c r="B2" s="3" t="n">
+        <v>46293.88350753472</v>
+      </c>
+      <c r="C2" s="7" t="inlineStr">
+        <is>
+          <t>דורש בדיקה</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>• שדה חובה חסר: מספר מסמך
+• שדה חובה חסר: תאריך המסמך
+• שדה חובה חסר: סה"כ לתשלום
+• שורה 3: אין סכום לשורה</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>מייל נכנס</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>גיא כהן &lt;mail4games21@gmail.com&gt;</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>בדיקת חשבונית (טסט לאוטומציה)</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>טופס התחשבנות 4 (תקול - חוסר שדות וערכים לא מספריים) - א.ב. מיזוג.pdf</t>
+        </is>
+      </c>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>א.ב. הנדסת מיזוג אוויר ואחזקת מבנים</t>
+        </is>
+      </c>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
+          <t>039481221</t>
+        </is>
+      </c>
+      <c r="K2" s="2" t="inlineStr">
+        <is>
+          <t>טופס התחשבנות זמני</t>
+        </is>
+      </c>
+      <c r="L2" s="2" t="n"/>
+      <c r="M2" s="5" t="n"/>
+      <c r="N2" s="5" t="n"/>
+      <c r="O2" s="5" t="n"/>
+      <c r="P2" s="2" t="inlineStr">
+        <is>
+          <t>ILS</t>
+        </is>
+      </c>
+      <c r="Q2" s="6" t="n">
+        <v>9550</v>
+      </c>
+      <c r="R2" s="2" t="n">
+        <v>17</v>
+      </c>
+      <c r="S2" s="6" t="n"/>
+      <c r="T2" s="6" t="n"/>
+      <c r="U2" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="V2" s="2" t="inlineStr">
+        <is>
+          <t>gemini/gemini-3.5-flash-lite</t>
+        </is>
+      </c>
+      <c r="W2" s="2" t="inlineStr">
+        <is>
+          <t>פרומפט מומלץ – טופסי התחשבנות v2</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="n">
+        <v>55</v>
+      </c>
+      <c r="B3" s="3" t="n">
+        <v>46293.88410210648</v>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>תקין</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr"/>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>מייל נכנס</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>גיא כהן &lt;mail4games21@gmail.com&gt;</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>בדיקת חשבונית (טסט לאוטומציה)</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>טופס התחשבנות 2 (תקין - עיצוב שונה) - ש.ל.ה הסעות רפואיות.pdf</t>
+        </is>
+      </c>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t>ש.ל.ה שירותי לוגיסטיקה והסעות רפואיות בע"מ</t>
+        </is>
+      </c>
+      <c r="J3" s="2" t="inlineStr">
+        <is>
+          <t>512998410</t>
+        </is>
+      </c>
+      <c r="K3" s="2" t="inlineStr">
+        <is>
+          <t>ריכוז חיובים חודשי / דרישת תשלום</t>
+        </is>
+      </c>
+      <c r="L3" s="2" t="inlineStr">
+        <is>
+          <t>SLH-88421</t>
+        </is>
+      </c>
+      <c r="M3" s="5" t="n">
+        <v>46264</v>
+      </c>
+      <c r="N3" s="5" t="n">
+        <v>46235</v>
+      </c>
+      <c r="O3" s="5" t="n">
+        <v>46265</v>
+      </c>
+      <c r="P3" s="2" t="inlineStr">
+        <is>
+          <t>ILS</t>
+        </is>
+      </c>
+      <c r="Q3" s="6" t="n">
+        <v>11000</v>
+      </c>
+      <c r="R3" s="2" t="n">
+        <v>17</v>
+      </c>
+      <c r="S3" s="6" t="n">
+        <v>1870</v>
+      </c>
+      <c r="T3" s="6" t="n">
+        <v>12870</v>
+      </c>
+      <c r="U3" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="V3" s="2" t="inlineStr">
+        <is>
+          <t>gemini/gemini-3.1-flash-lite</t>
+        </is>
+      </c>
+      <c r="W3" s="2" t="inlineStr">
+        <is>
+          <t>פרומפט מומלץ – טופסי התחשבנות v2</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="n">
+        <v>56</v>
+      </c>
+      <c r="B4" s="3" t="n">
+        <v>46293.88493513889</v>
+      </c>
+      <c r="C4" s="7" t="inlineStr">
+        <is>
+          <t>דורש בדיקה</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>• סכום השורות (14,100.00) שונה מהסה"כ לפני מע"מ (12,500.00)
+• סה"כ לפני מע"מ + מע"מ = 14,625.00, אך הסה"כ לתשלום בטופס הוא 15,625.00</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>מייל נכנס</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>גיא כהן &lt;mail4games21@gmail.com&gt;</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>בדיקת חשבונית (טסט לאוטומציה)</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>טופס התחשבנות 3 (תקול - אי התאמה בחישוב) - קלין-טק כביסה.pdf</t>
+        </is>
+      </c>
+      <c r="I4" s="2" t="inlineStr">
+        <is>
+          <t>קלין-טק שירותי כביסה וסטריליזציה למוסדות בע"מ</t>
+        </is>
+      </c>
+      <c r="J4" s="2" t="inlineStr">
+        <is>
+          <t>515602119</t>
+        </is>
+      </c>
+      <c r="K4" s="2" t="inlineStr">
+        <is>
+          <t>טופס התחשבנות</t>
+        </is>
+      </c>
+      <c r="L4" s="2" t="inlineStr">
+        <is>
+          <t>CT-2026-409</t>
+        </is>
+      </c>
+      <c r="M4" s="5" t="n">
+        <v>46275</v>
+      </c>
+      <c r="N4" s="5" t="n">
+        <v>46235</v>
+      </c>
+      <c r="O4" s="5" t="n">
+        <v>46265</v>
+      </c>
+      <c r="P4" s="2" t="inlineStr">
+        <is>
+          <t>ILS</t>
+        </is>
+      </c>
+      <c r="Q4" s="6" t="n">
+        <v>12500</v>
+      </c>
+      <c r="R4" s="2" t="n">
+        <v>17</v>
+      </c>
+      <c r="S4" s="6" t="n">
+        <v>2125</v>
+      </c>
+      <c r="T4" s="6" t="n">
+        <v>15625</v>
+      </c>
+      <c r="U4" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="V4" s="2" t="inlineStr">
+        <is>
+          <t>gemini/gemini-3.5-flash-lite</t>
+        </is>
+      </c>
+      <c r="W4" s="2" t="inlineStr">
+        <is>
+          <t>פרומפט מומלץ – טופסי התחשבנות v2</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="n">
+        <v>57</v>
+      </c>
+      <c r="B5" s="3" t="n">
+        <v>46293.88551366898</v>
+      </c>
+      <c r="C5" s="7" t="inlineStr">
+        <is>
+          <t>דורש בדיקה</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>• שורה 2: 250 × 16.00 = 4,000.00, אך בטופס מופיע 4,800.00
+• מע"מ 17% על 18,700.00 צריך להיות 3,179.00, אך בטופס מופיע 3,366.00</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>מייל נכנס</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>גיא כהן &lt;mail4games21@gmail.com&gt;</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>בדיקת חשבונית (טסט לאוטומציה)</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>טופס התחשבנות 5 (תקול - טעות כפל בשורה ומע_מ שגוי) - שפע קייטרינג.pdf</t>
+        </is>
+      </c>
+      <c r="I5" s="2" t="inlineStr">
+        <is>
+          <t>שפע טעמים - הסעדה וקייטרינג למוסדות רפואיים בע"מ</t>
+        </is>
+      </c>
+      <c r="J5" s="2" t="inlineStr">
+        <is>
+          <t>511209844</t>
+        </is>
+      </c>
+      <c r="K5" s="2" t="inlineStr">
+        <is>
+          <t>חשבונית ריכוז</t>
+        </is>
+      </c>
+      <c r="L5" s="2" t="inlineStr">
+        <is>
+          <t>SH-2026-9912</t>
+        </is>
+      </c>
+      <c r="M5" s="5" t="n">
+        <v>46267</v>
+      </c>
+      <c r="N5" s="5" t="n">
+        <v>46235</v>
+      </c>
+      <c r="O5" s="5" t="n">
+        <v>46265</v>
+      </c>
+      <c r="P5" s="2" t="inlineStr">
+        <is>
+          <t>ILS</t>
+        </is>
+      </c>
+      <c r="Q5" s="6" t="n">
+        <v>18700</v>
+      </c>
+      <c r="R5" s="2" t="n">
+        <v>17</v>
+      </c>
+      <c r="S5" s="6" t="n">
+        <v>3366</v>
+      </c>
+      <c r="T5" s="6" t="n">
+        <v>22066</v>
+      </c>
+      <c r="U5" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="V5" s="2" t="inlineStr">
+        <is>
+          <t>gemini/gemini-3.5-flash-lite</t>
+        </is>
+      </c>
+      <c r="W5" s="2" t="inlineStr">
+        <is>
+          <t>פרומפט מומלץ – טופסי התחשבנות v2</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="n">
+        <v>58</v>
+      </c>
+      <c r="B6" s="3" t="n">
+        <v>46293.88622248392</v>
+      </c>
+      <c r="C6" s="4" t="inlineStr">
+        <is>
+          <t>תקין</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr"/>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>מייל נכנס</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>גיא כהן &lt;mail4games21@gmail.com&gt;</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>בדיקת חשבונית (טסט לאוטומציה)</t>
+        </is>
+      </c>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t>טופס התחשבנות ספק - מדי-פארם בע_מ.pdf</t>
+        </is>
+      </c>
+      <c r="I6" s="2" t="inlineStr">
+        <is>
+          <t>מדי-פארם ציוד רפואי וסיעודי בע"מ</t>
+        </is>
+      </c>
+      <c r="J6" s="2" t="inlineStr">
+        <is>
+          <t>514892031</t>
+        </is>
+      </c>
+      <c r="K6" s="2" t="inlineStr">
+        <is>
+          <t>טופס התחשבנות ספק / חשבונית</t>
+        </is>
+      </c>
+      <c r="L6" s="2" t="inlineStr">
+        <is>
+          <t>MP-2026-0894</t>
+        </is>
+      </c>
+      <c r="M6" s="5" t="n">
+        <v>46280</v>
+      </c>
+      <c r="N6" s="5" t="n">
+        <v>46235</v>
+      </c>
+      <c r="O6" s="5" t="n">
+        <v>46265</v>
+      </c>
+      <c r="P6" s="2" t="inlineStr">
+        <is>
+          <t>ILS</t>
+        </is>
+      </c>
+      <c r="Q6" s="6" t="n">
+        <v>16000</v>
+      </c>
+      <c r="R6" s="2" t="n">
+        <v>17</v>
+      </c>
+      <c r="S6" s="6" t="n">
+        <v>2720</v>
+      </c>
+      <c r="T6" s="6" t="n">
+        <v>18720</v>
+      </c>
+      <c r="U6" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="V6" s="2" t="inlineStr">
+        <is>
+          <t>gemini/gemini-3.5-flash-lite</t>
+        </is>
+      </c>
+      <c r="W6" s="2" t="inlineStr">
+        <is>
+          <t>פרומפט מומלץ – טופסי התחשבנות v2</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:W1"/>
+  <autoFilter ref="A1:W6"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -586,7 +1087,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J1"/>
+  <dimension ref="A1:J18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -653,8 +1154,672 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" s="2" t="n">
+        <v>54</v>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>א.ב. הנדסת מיזוג אוויר ואחזקת מבנים</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="n"/>
+      <c r="D2" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E2" s="5" t="n">
+        <v>46237</v>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>החלפת מדחס מרכזי במערכת צ'ילר ראשית כולל פירוק והרכבה</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="H2" s="6" t="n">
+        <v>6400</v>
+      </c>
+      <c r="I2" s="6" t="n">
+        <v>6400</v>
+      </c>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
+          <t>תקין</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="n">
+        <v>54</v>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>א.ב. הנדסת מיזוג אוויר ואחזקת מבנים</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="n"/>
+      <c r="D3" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="E3" s="5" t="n">
+        <v>46245</v>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>ניקוי סוללות, שטיפת פילטרים וחיטוי תעלות ב35- חדרי אשפוז</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="n">
+        <v>35</v>
+      </c>
+      <c r="H3" s="6" t="n">
+        <v>90</v>
+      </c>
+      <c r="I3" s="6" t="n">
+        <v>3150</v>
+      </c>
+      <c r="J3" s="2" t="inlineStr">
+        <is>
+          <t>תקין</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="n">
+        <v>54</v>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>א.ב. הנדסת מיזוג אוויר ואחזקת מבנים</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="n"/>
+      <c r="D4" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="E4" s="5" t="n">
+        <v>46260</v>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>איתור דליפת גז בצנרת גג ומילוי גז פריאון A410R (לפי משקל)</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="H4" s="6" t="n"/>
+      <c r="I4" s="6" t="n"/>
+      <c r="J4" s="2" t="inlineStr">
+        <is>
+          <t>חסר סכום</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="n">
+        <v>55</v>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>ש.ל.ה שירותי לוגיסטיקה והסעות רפואיות בע"מ</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>SLH-88421</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E5" s="5" t="n">
+        <v>46239</v>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>הסעת מטופלים בכיסאות גלגלים (אמבולנס מותאם) קו מרכז גריאטרי גולדנקייר ← מרפאות חוץ שיבא תל השומר</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="n">
+        <v>18</v>
+      </c>
+      <c r="H5" s="6" t="n">
+        <v>350</v>
+      </c>
+      <c r="I5" s="6" t="n">
+        <v>6300</v>
+      </c>
+      <c r="J5" s="2" t="inlineStr">
+        <is>
+          <t>תקין</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="n">
+        <v>55</v>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>ש.ל.ה שירותי לוגיסטיקה והסעות רפואיות בע"מ</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>SLH-88421</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="E6" s="5" t="n">
+        <v>46248</v>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>שינוע דגימות מעבדה וציוד סטרילי בקירור (2–8 מעלות) איסוף יומי מרוכז מכלל מחלקות האשפוז והעברה למעבדה מרכזית</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="n">
+        <v>22</v>
+      </c>
+      <c r="H6" s="6" t="n">
+        <v>150</v>
+      </c>
+      <c r="I6" s="6" t="n">
+        <v>3300</v>
+      </c>
+      <c r="J6" s="2" t="inlineStr">
+        <is>
+          <t>תקין</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="n">
+        <v>55</v>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>ש.ל.ה שירותי לוגיסטיקה והסעות רפואיות בע"מ</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>SLH-88421</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="E7" s="5" t="n">
+        <v>46259</v>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>הזנקת חירום לילית – פינוי מטופל בליווי חובש כולל תוספת תעריף לילה והמתנת צוות רפואי בחדר מיון איכילוב</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="H7" s="6" t="n">
+        <v>700</v>
+      </c>
+      <c r="I7" s="6" t="n">
+        <v>1400</v>
+      </c>
+      <c r="J7" s="2" t="inlineStr">
+        <is>
+          <t>תקין</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="n">
+        <v>56</v>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>קלין-טק שירותי כביסה וסטריליזציה למוסדות בע"מ</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>CT-2026-409</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E8" s="5" t="n">
+        <v>46241</v>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>כביסה וחיטוי תרמי של מצעים, סדינים ומגבות (לפי משקל בק"ג)</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="n">
+        <v>1200</v>
+      </c>
+      <c r="H8" s="6" t="n">
+        <v>6.5</v>
+      </c>
+      <c r="I8" s="6" t="n">
+        <v>7800</v>
+      </c>
+      <c r="J8" s="2" t="inlineStr">
+        <is>
+          <t>תקין</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="n">
+        <v>56</v>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>קלין-טק שירותי כביסה וסטריליזציה למוסדות בע"מ</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>CT-2026-409</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="E9" s="5" t="n">
+        <v>46249</v>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>ניקוי יבש, חיטוי וגיהוץ מדי צוות רפואי וסיעודי (יחידות)</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="n">
+        <v>150</v>
+      </c>
+      <c r="H9" s="6" t="n">
+        <v>18</v>
+      </c>
+      <c r="I9" s="6" t="n">
+        <v>2700</v>
+      </c>
+      <c r="J9" s="2" t="inlineStr">
+        <is>
+          <t>תקין</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="n">
+        <v>56</v>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>קלין-טק שירותי כביסה וסטריליזציה למוסדות בע"מ</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>CT-2026-409</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="E10" s="5" t="n">
+        <v>46257</v>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>טיפול מיוחד בכביסה מזוהמת ואריזת ואקום לחדרי בידוד</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="n">
+        <v>80</v>
+      </c>
+      <c r="H10" s="6" t="n">
+        <v>25</v>
+      </c>
+      <c r="I10" s="6" t="n">
+        <v>2000</v>
+      </c>
+      <c r="J10" s="2" t="inlineStr">
+        <is>
+          <t>תקין</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="n">
+        <v>56</v>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>קלין-טק שירותי כביסה וסטריליזציה למוסדות בע"מ</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>CT-2026-409</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="E11" s="5" t="n">
+        <v>46265</v>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>דמי הובלה, איסוף והפצה שבועיים במשאית ייעודית (4 סבבים)</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="H11" s="6" t="n">
+        <v>400</v>
+      </c>
+      <c r="I11" s="6" t="n">
+        <v>1600</v>
+      </c>
+      <c r="J11" s="2" t="inlineStr">
+        <is>
+          <t>תקין</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="n">
+        <v>57</v>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>שפע טעמים - הסעדה וקייטרינג למוסדות רפואיים בע"מ</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>SH-2026-9912</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E12" s="5" t="n">
+        <v>46244</v>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>מנות צהריים חמות מותאמות (דל נתרן / מרקם טחון) - עשרת ראשונה</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="n">
+        <v>400</v>
+      </c>
+      <c r="H12" s="6" t="n">
+        <v>28</v>
+      </c>
+      <c r="I12" s="6" t="n">
+        <v>11200</v>
+      </c>
+      <c r="J12" s="2" t="inlineStr">
+        <is>
+          <t>תקין</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="n">
+        <v>57</v>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>שפע טעמים - הסעדה וקייטרינג למוסדות רפואיים בע"מ</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>SH-2026-9912</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="E13" s="5" t="n">
+        <v>46254</v>
+      </c>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>מארזי ארוחות בוקר וערב אישיים למחלקת שיקום ותשושי נפש</t>
+        </is>
+      </c>
+      <c r="G13" s="2" t="n">
+        <v>250</v>
+      </c>
+      <c r="H13" s="6" t="n">
+        <v>16</v>
+      </c>
+      <c r="I13" s="6" t="n">
+        <v>4800</v>
+      </c>
+      <c r="J13" s="2" t="inlineStr">
+        <is>
+          <t>שגיאת חישוב</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="n">
+        <v>57</v>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>שפע טעמים - הסעדה וקייטרינג למוסדות רפואיים בע"מ</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>SH-2026-9912</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="E14" s="5" t="n">
+        <v>46265</v>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>אספקת פורמולות העשרה תזונתית ואבקות חלבון קליניות</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="n">
+        <v>60</v>
+      </c>
+      <c r="H14" s="6" t="n">
+        <v>45</v>
+      </c>
+      <c r="I14" s="6" t="n">
+        <v>2700</v>
+      </c>
+      <c r="J14" s="2" t="inlineStr">
+        <is>
+          <t>תקין</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="n">
+        <v>58</v>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>מדי-פארם ציוד רפואי וסיעודי בע"מ</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>MP-2026-0894</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E15" s="5" t="n">
+        <v>46238</v>
+      </c>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t>ערכות ציוד סיעודי מתכלה – אספקה חודשית מרוכזת תעודת משלוח מס' 88412 | חלוקה למחלקות א'–ג'</t>
+        </is>
+      </c>
+      <c r="G15" s="2" t="n">
+        <v>25</v>
+      </c>
+      <c r="H15" s="6" t="n">
+        <v>320</v>
+      </c>
+      <c r="I15" s="6" t="n">
+        <v>8000</v>
+      </c>
+      <c r="J15" s="2" t="inlineStr">
+        <is>
+          <t>תקין</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="n">
+        <v>58</v>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>מדי-פארם ציוד רפואי וסיעודי בע"מ</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>MP-2026-0894</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="E16" s="5" t="n">
+        <v>46246</v>
+      </c>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t>תחזוקה תקופתית וכיול מכשירי ניטור ומדדי לחץ דם קריאת שירות מרוכזת מס' 4190 | כולל הנפקת תעודות תקינות</t>
+        </is>
+      </c>
+      <c r="G16" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="H16" s="6" t="n">
+        <v>250</v>
+      </c>
+      <c r="I16" s="6" t="n">
+        <v>3000</v>
+      </c>
+      <c r="J16" s="2" t="inlineStr">
+        <is>
+          <t>תקין</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="n">
+        <v>58</v>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>מדי-פארם ציוד רפואי וסיעודי בע"מ</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>MP-2026-0894</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="E17" s="5" t="n">
+        <v>46254</v>
+      </c>
+      <c r="F17" s="2" t="inlineStr">
+        <is>
+          <t>השכרת מיטות סיעודיות חשמליות ומזרני לחץ דינמיים חיוב שכירות חודשי קבוע עבור חודש אוגוסט 2026</t>
+        </is>
+      </c>
+      <c r="G17" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="H17" s="6" t="n">
+        <v>450</v>
+      </c>
+      <c r="I17" s="6" t="n">
+        <v>3600</v>
+      </c>
+      <c r="J17" s="2" t="inlineStr">
+        <is>
+          <t>תקין</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="n">
+        <v>58</v>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>מדי-פארם ציוד רפואי וסיעודי בע"מ</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>MP-2026-0894</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="E18" s="5" t="n">
+        <v>46262</v>
+      </c>
+      <c r="F18" s="2" t="inlineStr">
+        <is>
+          <t>מילוי ואספקה דחופה של מחוללי ובלוני חמצן ניידים תעודת משלוח מס' 88905 | כולל בדיקת וסתים בטיחותית</t>
+        </is>
+      </c>
+      <c r="G18" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="H18" s="6" t="n">
+        <v>280</v>
+      </c>
+      <c r="I18" s="6" t="n">
+        <v>1400</v>
+      </c>
+      <c r="J18" s="2" t="inlineStr">
+        <is>
+          <t>תקין</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J1"/>
+  <autoFilter ref="A1:J18"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>